<commit_message>
Complete Audi repair-first fitment review
</commit_message>
<xml_diff>
--- a/outputs/audi-repair-first-review/Audi-repair-first-fitment-review.xlsx
+++ b/outputs/audi-repair-first-review/Audi-repair-first-fitment-review.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re236912b51844fae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audi Review" sheetId="2" r:id="Re5774462ba8747fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="Rf8f873359b384a8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R5e7c561b84ab4128"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8d564973ed8a4154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audi Review" sheetId="2" r:id="R8d81e17349944e77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Remaining Queue" sheetId="3" r:id="R28856ca671bf4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R5964678d3fbb4ac3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -90,7 +90,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left/>
@@ -120,11 +120,25 @@
       <x:right/>
       <x:bottom/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
+    <x:border>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="50">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +229,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
@@ -484,7 +507,7 @@
         <x:v>Reviewed in this batch</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>350</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="C5" s="11"/>
       <x:c r="D5" s="11"/>
@@ -498,7 +521,7 @@
         <x:v>Remaining queue</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
-        <x:v>39</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="11"/>
       <x:c r="D6" s="11"/>
@@ -512,7 +535,7 @@
         <x:v>Issues with destinations</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
-        <x:v>344</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="C7" s="11"/>
       <x:c r="D7" s="11"/>
@@ -526,7 +549,7 @@
         <x:v>Destination entries</x:v>
       </x:c>
       <x:c r="B8" s="13" t="n">
-        <x:v>603</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="C8" s="11"/>
       <x:c r="D8" s="11"/>
@@ -540,7 +563,7 @@
         <x:v>Distinct URLs</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
-        <x:v>101</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C9" s="11"/>
       <x:c r="D9" s="11"/>
@@ -21563,46 +21586,2380 @@
       <x:c r="N609" s="41" t="str"/>
     </x:row>
     <x:row r="610" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A610" s="42" t="n">
+      <x:c r="A610" s="40" t="n">
         <x:v>350</x:v>
       </x:c>
-      <x:c r="B610" s="43" t="str">
+      <x:c r="B610" s="9" t="str">
         <x:v>audi-sq2-ea888-2-0-tfsi-coolant-leak-from-water-pump-thermostat-housi</x:v>
       </x:c>
-      <x:c r="C610" s="43" t="str">
+      <x:c r="C610" s="9" t="str">
         <x:v>2019-2024 | Audi | SQ2 | 2.0 TFSI quattro | EA888 2.0 TFSI Gen3</x:v>
       </x:c>
-      <x:c r="D610" s="43" t="str">
+      <x:c r="D610" s="9" t="str">
         <x:v>EA888 2.0 TFSI coolant leak from water pump / thermostat housing</x:v>
       </x:c>
-      <x:c r="E610" s="43" t="str">
+      <x:c r="E610" s="9" t="str">
         <x:v>Replace the failed water pump / thermostat housing assembly, ideally with the latest revised, more heat-resistant unit; many shops fit an upgraded repair kit and a new gasket. Catch it early by watching for slowly dropping coolant level and a faint sweet smell. Combine with a coolant flush and refill.</x:v>
       </x:c>
-      <x:c r="F610" s="43" t="str">
+      <x:c r="F610" s="9" t="str">
         <x:v>Non-US-market engine/VIN pressure test; exact pump/thermostat/housing leak source and revision; gasket/coolant/bleed</x:v>
       </x:c>
-      <x:c r="G610" s="43" t="str">
+      <x:c r="G610" s="9" t="str">
         <x:v>NON-US-MARKET / LEAK-SOURCE GATE</x:v>
       </x:c>
-      <x:c r="H610" s="43" t="str">
+      <x:c r="H610" s="9" t="str">
         <x:v>Audi UK service and maintenance</x:v>
       </x:c>
-      <x:c r="I610" s="43" t="str">
+      <x:c r="I610" s="9" t="str">
         <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
       </x:c>
-      <x:c r="J610" s="43" t="str">
+      <x:c r="J610" s="9" t="str">
         <x:v>2019-2024 SQ2 local-market EA888 coolant diagnosis</x:v>
       </x:c>
-      <x:c r="K610" s="43" t="str">
+      <x:c r="K610" s="9" t="str">
         <x:v>manufacturer-market service</x:v>
       </x:c>
-      <x:c r="L610" s="43" t="str"/>
-      <x:c r="M610" s="43" t="str">
+      <x:c r="L610" s="9" t="str"/>
+      <x:c r="M610" s="9" t="str">
         <x:v>SQ2 is non-US and exact assembly/revision requires market VIN.</x:v>
       </x:c>
-      <x:c r="N610" s="44" t="str">
+      <x:c r="N610" s="41" t="str">
         <x:v>No US affiliate or generic upgraded kit; do not bundle flush automatically.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="611" ht="396" hidden="0" customHeight="1">
+      <x:c r="A611" s="40" t="n">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B611" s="9" t="str">
+        <x:v>audi-sq2-electro-mechanical-parking-brake-brake-pedal-weld-recalls</x:v>
+      </x:c>
+      <x:c r="C611" s="9" t="str">
+        <x:v>2019-2020 | Audi | SQ2</x:v>
+      </x:c>
+      <x:c r="D611" s="9" t="str">
+        <x:v>Electro-mechanical parking brake and brake-pedal weld recalls (early build)</x:v>
+      </x:c>
+      <x:c r="E611" s="9" t="str">
+        <x:v>These are recall items — have the VIN checked against the Audi/DVSA recall database and any open campaign rectified free of charge at a dealer. Report any abnormal parking-brake behaviour or a soft/abnormal brake pedal immediately.</x:v>
+      </x:c>
+      <x:c r="F611" s="9" t="str">
+        <x:v>Local-market VIN recall check; dealer parking-brake and brake-pedal campaign remedy; urgent inspection for abnormal operation</x:v>
+      </x:c>
+      <x:c r="G611" s="9" t="str">
+        <x:v>NON-US RECALL ROUTE</x:v>
+      </x:c>
+      <x:c r="H611" s="9" t="str">
+        <x:v>Audi UK service and maintenance</x:v>
+      </x:c>
+      <x:c r="I611" s="9" t="str">
+        <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
+      </x:c>
+      <x:c r="J611" s="9" t="str">
+        <x:v>2019-2020 SQ2 local-market recall/VIN check</x:v>
+      </x:c>
+      <x:c r="K611" s="9" t="str">
+        <x:v>manufacturer-market campaign service</x:v>
+      </x:c>
+      <x:c r="L611" s="9" t="str"/>
+      <x:c r="M611" s="9" t="str">
+        <x:v>Safety campaign remedy is dealer-controlled and market/VIN specific.</x:v>
+      </x:c>
+      <x:c r="N611" s="41" t="str">
+        <x:v>No parking-brake module or pedal product link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="612" ht="475.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A612" s="40" t="n">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="B612" s="9" t="str">
+        <x:v>audi-sq2-internal-fuse-box-wiring-harness-can-work-loose-causing-sudd</x:v>
+      </x:c>
+      <x:c r="C612" s="9" t="str">
+        <x:v>2022-2023 | Audi | SQ2 | 2.0 TFSI</x:v>
+      </x:c>
+      <x:c r="D612" s="9" t="str">
+        <x:v>2022-2023 Audi SQ2 Interior Fuse-Carrier Recall GAI-3692</x:v>
+      </x:c>
+      <x:c r="E612" s="9" t="str">
+        <x:v>Check the VIN and open-campaign status with an authorised Audi dealer in the vehicle’s market. The campaign remedy is dealer inspection and correction of the fuse-carrier power connection. Do not replace a fuse box or wiring harness solely from a warning lamp or this model-year summary.</x:v>
+      </x:c>
+      <x:c r="F612" s="9" t="str">
+        <x:v>Local-market VIN/GAI-3692 check; dealer fuse-carrier inspection and campaign correction</x:v>
+      </x:c>
+      <x:c r="G612" s="9" t="str">
+        <x:v>NON-US RECALL ROUTE</x:v>
+      </x:c>
+      <x:c r="H612" s="9" t="str">
+        <x:v>Audi UK service and maintenance</x:v>
+      </x:c>
+      <x:c r="I612" s="9" t="str">
+        <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
+      </x:c>
+      <x:c r="J612" s="9" t="str">
+        <x:v>2022-2023 SQ2 local-market fuse-carrier campaign</x:v>
+      </x:c>
+      <x:c r="K612" s="9" t="str">
+        <x:v>manufacturer-market campaign service</x:v>
+      </x:c>
+      <x:c r="L612" s="9" t="str"/>
+      <x:c r="M612" s="9" t="str">
+        <x:v>The campaign defines the inspection/correction.</x:v>
+      </x:c>
+      <x:c r="N612" s="41" t="str">
+        <x:v>No fuse box or harness product link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="613" ht="488.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A613" s="40" t="n">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B613" s="9" t="str">
+        <x:v>audi-sq2-mmi-infotainment-freezing-rebooting-lost-settings</x:v>
+      </x:c>
+      <x:c r="C613" s="9" t="str">
+        <x:v>2019-2024 | Audi | SQ2</x:v>
+      </x:c>
+      <x:c r="D613" s="9" t="str">
+        <x:v>MMI infotainment freezing, rebooting and lost settings</x:v>
+      </x:c>
+      <x:c r="E613" s="9" t="str">
+        <x:v>A forced MMI restart (press and hold the on/off or volume control ~10 seconds until it reboots) clears many transient faults. Persistent issues are usually resolved by a dealer software/firmware update; check for any applicable MMI update campaigns. Only in rare cases is the MMI head unit itself replaced.</x:v>
+      </x:c>
+      <x:c r="F613" s="9" t="str">
+        <x:v>Safe restart; local-market software/version diagnosis; head unit only after hardware failure is proven</x:v>
+      </x:c>
+      <x:c r="G613" s="9" t="str">
+        <x:v>NON-US SOFTWARE-FIRST SERVICE</x:v>
+      </x:c>
+      <x:c r="H613" s="9" t="str">
+        <x:v>Audi UK service and maintenance</x:v>
+      </x:c>
+      <x:c r="I613" s="9" t="str">
+        <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
+      </x:c>
+      <x:c r="J613" s="9" t="str">
+        <x:v>2019-2024 SQ2 MMI software and hardware diagnosis</x:v>
+      </x:c>
+      <x:c r="K613" s="9" t="str">
+        <x:v>manufacturer-market service</x:v>
+      </x:c>
+      <x:c r="L613" s="9" t="str"/>
+      <x:c r="M613" s="9" t="str">
+        <x:v>Rebooting does not establish a failed head unit.</x:v>
+      </x:c>
+      <x:c r="N613" s="41" t="str">
+        <x:v>No generic module or scanner link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="614" ht="488.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A614" s="40" t="n">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B614" s="9" t="str">
+        <x:v>audi-sq2-pcv-crankcase-ventilation-valve-diaphragm-failure-causing-ro</x:v>
+      </x:c>
+      <x:c r="C614" s="9" t="str">
+        <x:v>2019-2024 | Audi | SQ2 | EA888 2.0 TFSI Gen3</x:v>
+      </x:c>
+      <x:c r="D614" s="9" t="str">
+        <x:v>PCV / crankcase ventilation valve diaphragm failure causing rough idle and lean-running codes</x:v>
+      </x:c>
+      <x:c r="E614" s="9" t="str">
+        <x:v>Replace the PCV valve (or the valve-cover assembly that integrates it) with the latest revised part; some owners fit a catch-can to reduce recurrence. A quick field test — briefly covering the bleeder hole on the cap to see if idle stabilises or whistling stops — helps confirm before replacement.</x:v>
+      </x:c>
+      <x:c r="F614" s="9" t="str">
+        <x:v>Measured crankcase vacuum and intake/smoke diagnosis; exact engine/VIN PCV valve or valve-cover assembly only after proof</x:v>
+      </x:c>
+      <x:c r="G614" s="9" t="str">
+        <x:v>NON-US ENGINE / PCV DIAGNOSIS GATE</x:v>
+      </x:c>
+      <x:c r="H614" s="9" t="str">
+        <x:v>Audi UK service and maintenance</x:v>
+      </x:c>
+      <x:c r="I614" s="9" t="str">
+        <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
+      </x:c>
+      <x:c r="J614" s="9" t="str">
+        <x:v>2019-2024 SQ2 engine-specific crankcase diagnosis</x:v>
+      </x:c>
+      <x:c r="K614" s="9" t="str">
+        <x:v>manufacturer-market service</x:v>
+      </x:c>
+      <x:c r="L614" s="9" t="str"/>
+      <x:c r="M614" s="9" t="str">
+        <x:v>Oil-cap feel alone cannot select a valve or complete cover.</x:v>
+      </x:c>
+      <x:c r="N614" s="41" t="str">
+        <x:v>No catch-can prevention claim or universal cover replacement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="615" ht="752.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A615" s="40" t="n">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B615" s="9" t="str">
+        <x:v>audi-sq2-s-tronic-7-speed-wet-clutch-transmission-jerky-low-speed-shi</x:v>
+      </x:c>
+      <x:c r="C615" s="9" t="str">
+        <x:v>2019-2024 | Audi | SQ2 | 7-speed S tronic | DQ381 / 0GC 7-speed wet-clutch S tronic</x:v>
+      </x:c>
+      <x:c r="D615" s="9" t="str">
+        <x:v>S tronic (DQ381) 7-speed wet-clutch transmission: jerky low-speed shifts, hesitation and limp mode</x:v>
+      </x:c>
+      <x:c r="E615" s="9" t="str">
+        <x:v>First step is a proper DSG fluid-and-filter service (the wet-clutch unit needs periodic transmission oil changes — many owners do it around 40k miles even though intervals can be longer). Have the TCU scanned for stored codes; sensor or mechatronic valve replacement and re-coding/adaptation resolves many cases, while severe cases need a full mechatronic unit or clutch-pack replacement. Insist on a software/adaptation update at the dealer for driveability complaints.</x:v>
+      </x:c>
+      <x:c r="F615" s="9" t="str">
+        <x:v>Confirm DQ381/0GC code; faults/fluid condition; exact market service schedule; software/adaptation; mechatronic or clutch only by test</x:v>
+      </x:c>
+      <x:c r="G615" s="9" t="str">
+        <x:v>NON-US TRANSMISSION-CODE / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H615" s="9" t="str">
+        <x:v>Audi UK service and maintenance</x:v>
+      </x:c>
+      <x:c r="I615" s="9" t="str">
+        <x:v>https://www.audi.co.uk/en/owners/service-and-maintenance/</x:v>
+      </x:c>
+      <x:c r="J615" s="9" t="str">
+        <x:v>2019-2024 SQ2 transmission-code service and diagnosis</x:v>
+      </x:c>
+      <x:c r="K615" s="9" t="str">
+        <x:v>manufacturer-market service</x:v>
+      </x:c>
+      <x:c r="L615" s="9" t="str"/>
+      <x:c r="M615" s="9" t="str">
+        <x:v>Service, software, mechatronic and clutch are different branches.</x:v>
+      </x:c>
+      <x:c r="N615" s="41" t="str">
+        <x:v>No generic DSG kit or fixed interval without exact local manual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="616" ht="541.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A616" s="40" t="n">
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="B616" s="9" t="str">
+        <x:v>audi-sq5-air-suspension-2018</x:v>
+      </x:c>
+      <x:c r="C616" s="9" t="str">
+        <x:v>2018-2025 | Audi | SQ5</x:v>
+      </x:c>
+      <x:c r="D616" s="9" t="str">
+        <x:v>Air-Suspension Warning with C1260F0 or U112100 Communication Fault</x:v>
+      </x:c>
+      <x:c r="E616" s="9" t="str">
+        <x:v>Inspect the wiring and connector contacts between J775 and J1135 first. If no wiring fault is found, clear a first passive or sporadic fault and release the vehicle. Replace J1135 for an active or static fault, or when the same passive or sporadic fault returns a second time, following Audi workshop information and VIN-specific ETKA data.</x:v>
+      </x:c>
+      <x:c r="F616" s="9" t="str">
+        <x:v>J775-J1135 wiring/contact inspection; occurrence-state logic; J1135 only after active/static or repeated passive fault</x:v>
+      </x:c>
+      <x:c r="G616" s="9" t="str">
+        <x:v>WIRING-FIRST TSB / CONTROL-UNIT GATE</x:v>
+      </x:c>
+      <x:c r="H616" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I616" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J616" s="9" t="str">
+        <x:v>2018-2025 SQ5 J1135 guided diagnosis</x:v>
+      </x:c>
+      <x:c r="K616" s="9" t="str">
+        <x:v>manufacturer suspension service</x:v>
+      </x:c>
+      <x:c r="L616" s="9" t="str"/>
+      <x:c r="M616" s="9" t="str">
+        <x:v>The procedure does not establish a failed strut or compressor.</x:v>
+      </x:c>
+      <x:c r="N616" s="41" t="str">
+        <x:v>No air-suspension hardware link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="617" ht="924" hidden="0" customHeight="1">
+      <x:c r="A617" s="40" t="n">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="B617" s="9" t="str">
+        <x:v>audi-sq5-carbon-buildup-2014</x:v>
+      </x:c>
+      <x:c r="C617" s="9" t="str">
+        <x:v>2014-2025 | Audi | SQ5 | 3.0T Supercharged, 3.0T</x:v>
+      </x:c>
+      <x:c r="D617" s="9" t="str">
+        <x:v>Fuel-Quality or Deposit-Related Rough Running and Misfire Diagnosis</x:v>
+      </x:c>
+      <x:c r="E617" s="9" t="str">
+        <x:v>Confirm fuel quality, symptoms and stored DTCs before replacing or cleaning components. If contaminated gasoline is suspected, advise changing the fuel source; if low detergent quality is suspected, Audi recommends Top Tier detergent gasoline. Continue workshop diagnosis if symptoms persist. On 2018-2025 EA839 SQ5 models, do not recommend unapproved cleaners or additives; follow the owner manual and use only Audi-approved petrol additives. Do not prescribe routine walnut blasting, a catch can or chemical cleaning from this record.</x:v>
+      </x:c>
+      <x:c r="F617" s="9" t="str">
+        <x:v>Split supercharged/turbo engines; ignition/fuel/air diagnosis before deposit confirmation; use detergent-standard gasoline</x:v>
+      </x:c>
+      <x:c r="G617" s="9" t="str">
+        <x:v>ENGINE-GENERATION / DIAGNOSIS GATE</x:v>
+      </x:c>
+      <x:c r="H617" s="9" t="str">
+        <x:v>TOP TIER gasoline stations</x:v>
+      </x:c>
+      <x:c r="I617" s="9" t="str">
+        <x:v>https://www.toptiergas.com/gasoline-brands/</x:v>
+      </x:c>
+      <x:c r="J617" s="9" t="str">
+        <x:v>2014-2025 SQ5 fuel-quality maintenance</x:v>
+      </x:c>
+      <x:c r="K617" s="9" t="str">
+        <x:v>standards-based fuel locator</x:v>
+      </x:c>
+      <x:c r="L617" s="9" t="str"/>
+      <x:c r="M617" s="9" t="str">
+        <x:v>The range spans different engines and symptoms do not prove deposits.</x:v>
+      </x:c>
+      <x:c r="N617" s="41" t="str">
+        <x:v>No walnut blasting, additive or catch-can link before confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="618" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A618" s="40" t="str"/>
+      <x:c r="B618" s="9" t="str"/>
+      <x:c r="C618" s="9" t="str"/>
+      <x:c r="D618" s="9" t="str"/>
+      <x:c r="E618" s="9" t="str"/>
+      <x:c r="F618" s="9" t="str"/>
+      <x:c r="G618" s="9" t="str"/>
+      <x:c r="H618" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I618" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J618" s="9" t="str">
+        <x:v>SQ5 engine-specific rough-running/deposit diagnosis</x:v>
+      </x:c>
+      <x:c r="K618" s="9" t="str">
+        <x:v>specialist intake service</x:v>
+      </x:c>
+      <x:c r="L618" s="9" t="str"/>
+      <x:c r="M618" s="9" t="str"/>
+      <x:c r="N618" s="41" t="str"/>
+    </x:row>
+    <x:row r="619" ht="765.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A619" s="40" t="n">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B619" s="9" t="str">
+        <x:v>audi-sq5-pcv-valve-2014</x:v>
+      </x:c>
+      <x:c r="C619" s="9" t="str">
+        <x:v>2014-2017 | Audi | SQ5 | 3.0T Supercharged</x:v>
+      </x:c>
+      <x:c r="D619" s="9" t="str">
+        <x:v>P052E00 Crankcase-Breather Membrane or Elbow Fault</x:v>
+      </x:c>
+      <x:c r="E619" s="9" t="str">
+        <x:v>Use Audi hand-vacuum test to distinguish a membrane leak from an elbow fault. If indicated, remove the compressor or intake manifold and inspect the membrane and the breather two metal plates. Use repair kit 06E103772H only for a confirmed membrane or plate fault. For a confirmed elbow fault, replace elbow 06E103402 and spring clip N10769401 rather than automatically replacing the complete breather. Verify current part data in ETKA before ordering.</x:v>
+      </x:c>
+      <x:c r="F619" s="9" t="str">
+        <x:v>Hand-vacuum test of membrane versus breather elbow; exact engine/VIN 06E103772H repair kit or 06E103402 elbow plus N10769401 clip by branch</x:v>
+      </x:c>
+      <x:c r="G619" s="9" t="str">
+        <x:v>SUPERCHARGED ENGINE / TEST-BRANCH GATE</x:v>
+      </x:c>
+      <x:c r="H619" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I619" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J619" s="9" t="str">
+        <x:v>2014-2017 SQ5 VIN-specific PCV membrane/elbow parts</x:v>
+      </x:c>
+      <x:c r="K619" s="9" t="str">
+        <x:v>manufacturer parts route</x:v>
+      </x:c>
+      <x:c r="L619" s="9" t="str"/>
+      <x:c r="M619" s="9" t="str">
+        <x:v>Membrane and elbow failures require different parts.</x:v>
+      </x:c>
+      <x:c r="N619" s="41" t="str">
+        <x:v>Hold retail kit until live fitment and contents are verified for VIN.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="620" ht="66" hidden="0" customHeight="1">
+      <x:c r="A620" s="40" t="str"/>
+      <x:c r="B620" s="9" t="str"/>
+      <x:c r="C620" s="9" t="str"/>
+      <x:c r="D620" s="9" t="str"/>
+      <x:c r="E620" s="9" t="str"/>
+      <x:c r="F620" s="9" t="str"/>
+      <x:c r="G620" s="9" t="str"/>
+      <x:c r="H620" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I620" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J620" s="9" t="str">
+        <x:v>vacuum test and branch-specific repair</x:v>
+      </x:c>
+      <x:c r="K620" s="9" t="str">
+        <x:v>specialist engine service</x:v>
+      </x:c>
+      <x:c r="L620" s="9" t="str"/>
+      <x:c r="M620" s="9" t="str"/>
+      <x:c r="N620" s="41" t="str"/>
+    </x:row>
+    <x:row r="621" ht="250.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A621" s="40" t="n">
+        <x:v>359</x:v>
+      </x:c>
+      <x:c r="B621" s="9" t="str">
+        <x:v>audi-sq5-supercharger-2014</x:v>
+      </x:c>
+      <x:c r="C621" s="9" t="str">
+        <x:v>2014-2018 | Audi | SQ5 | 3.0T</x:v>
+      </x:c>
+      <x:c r="D621" s="9" t="str">
+        <x:v>3.0T Supercharger Bearing and Intercooler Pump Failure</x:v>
+      </x:c>
+      <x:c r="E621" s="9" t="str">
+        <x:v>Replace supercharger nose bearing kit. Replace intercooler pump if failing. Service supercharger belt tension.</x:v>
+      </x:c>
+      <x:c r="F621" s="9" t="str">
+        <x:v>Correct generation; diagnose accessory drive, supercharger nose/clutch and charge-cooling circuit separately; exact component only after proof</x:v>
+      </x:c>
+      <x:c r="G621" s="9" t="str">
+        <x:v>SOURCE RANGE ERROR / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H621" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I621" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J621" s="9" t="str">
+        <x:v>2014-2017 supercharged SQ5 noise/cooling diagnosis</x:v>
+      </x:c>
+      <x:c r="K621" s="9" t="str">
+        <x:v>specialist engine service</x:v>
+      </x:c>
+      <x:c r="L621" s="9" t="str"/>
+      <x:c r="M621" s="9" t="str">
+        <x:v>2018 SQ5 uses a turbocharged EA839, not the described supercharger.</x:v>
+      </x:c>
+      <x:c r="N621" s="41" t="str">
+        <x:v>No supercharger kit, pump or belt until generation and failed component are corrected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="622" ht="66" hidden="0" customHeight="1">
+      <x:c r="A622" s="40" t="str"/>
+      <x:c r="B622" s="9" t="str"/>
+      <x:c r="C622" s="9" t="str"/>
+      <x:c r="D622" s="9" t="str"/>
+      <x:c r="E622" s="9" t="str"/>
+      <x:c r="F622" s="9" t="str"/>
+      <x:c r="G622" s="9" t="str"/>
+      <x:c r="H622" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I622" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J622" s="9" t="str">
+        <x:v>VIN component/procedure</x:v>
+      </x:c>
+      <x:c r="K622" s="9" t="str">
+        <x:v>manufacturer parts route</x:v>
+      </x:c>
+      <x:c r="L622" s="9" t="str"/>
+      <x:c r="M622" s="9" t="str"/>
+      <x:c r="N622" s="41" t="str"/>
+    </x:row>
+    <x:row r="623" ht="844.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A623" s="40" t="n">
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="B623" s="9" t="str">
+        <x:v>audi-sq5-supercharger-oil-leak-2014</x:v>
+      </x:c>
+      <x:c r="C623" s="9" t="str">
+        <x:v>2014-2017 | Audi | SQ5 | Premium Plus, Prestige | 3.0T Supercharged, 3.0T</x:v>
+      </x:c>
+      <x:c r="D623" s="9" t="str">
+        <x:v>Supercharger Seal and Gasket Oil Leaks (3.0T)</x:v>
+      </x:c>
+      <x:c r="E623" s="9" t="str">
+        <x:v>JHM Motorsports sells a complete supercharger replacement seal and gasket kit for the Eaton unit in the 3.0T. Replacing all seals at once is recommended since the supercharger must be removed for access. Nose cone seal, rotor shaft seals, and manifold gaskets should all be replaced together ($300-$500 in parts, $600-$1,200 labor). While the supercharger is off, also replace the PCV valve and perform carbon cleaning. For valve cover gasket leaks (separate issue), budget $400-$800 parts and labor. Monitor oil level weekly if leaks are present.</x:v>
+      </x:c>
+      <x:c r="F623" s="9" t="str">
+        <x:v>Clean and trace exact supercharger/engine leak; engine-specific seal scope; PCV and intake deposits only as separate confirmed work</x:v>
+      </x:c>
+      <x:c r="G623" s="9" t="str">
+        <x:v>LEAK-SOURCE / ENGINE GATE</x:v>
+      </x:c>
+      <x:c r="H623" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I623" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J623" s="9" t="str">
+        <x:v>2014-2017 SQ5 supercharger leak diagnosis/reseal</x:v>
+      </x:c>
+      <x:c r="K623" s="9" t="str">
+        <x:v>specialist engine service</x:v>
+      </x:c>
+      <x:c r="L623" s="9" t="str"/>
+      <x:c r="M623" s="9" t="str">
+        <x:v>A complete aftermarket seal kit and all overlapping work were not proven necessary.</x:v>
+      </x:c>
+      <x:c r="N623" s="41" t="str">
+        <x:v>Hold JHM kit until the live page proves SQ5 engine fitment and complete contents.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="624" ht="66" hidden="0" customHeight="1">
+      <x:c r="A624" s="40" t="str"/>
+      <x:c r="B624" s="9" t="str"/>
+      <x:c r="C624" s="9" t="str"/>
+      <x:c r="D624" s="9" t="str"/>
+      <x:c r="E624" s="9" t="str"/>
+      <x:c r="F624" s="9" t="str"/>
+      <x:c r="G624" s="9" t="str"/>
+      <x:c r="H624" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I624" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J624" s="9" t="str">
+        <x:v>VIN seal diagrams and parts</x:v>
+      </x:c>
+      <x:c r="K624" s="9" t="str">
+        <x:v>manufacturer parts route</x:v>
+      </x:c>
+      <x:c r="L624" s="9" t="str"/>
+      <x:c r="M624" s="9" t="str"/>
+      <x:c r="N624" s="41" t="str"/>
+    </x:row>
+    <x:row r="625" ht="1122" hidden="0" customHeight="1">
+      <x:c r="A625" s="40" t="n">
+        <x:v>361</x:v>
+      </x:c>
+      <x:c r="B625" s="9" t="str">
+        <x:v>audi-sq5-water-pump-2018</x:v>
+      </x:c>
+      <x:c r="C625" s="9" t="str">
+        <x:v>2018-2024 | Audi | SQ5 | 3.0T</x:v>
+      </x:c>
+      <x:c r="D625" s="9" t="str">
+        <x:v>Mechanical Coolant-Pump Leak with Possible N649 Vacuum-System Contamination</x:v>
+      </x:c>
+      <x:c r="E625" s="9" t="str">
+        <x:v>Confirm the complaint and exact vehicle criteria first. Inspect the vacuum line and N649 for coolant, then clean and dry suspected leakage, fill the cooling system correctly, inspect at idle and around 2,500 rpm, and pressure-test according to Audi workshop information. If no leak is reproduced, observe the vehicle without replacing parts. If the pump leak is confirmed, replace the failed component and document it. If fresh coolant has entered the vacuum system, inspect the remaining Audi checkpoints and replace only contaminated components; if the downstream checkpoints are clean, replace N649 and clean the line between the pump and N649 as directed by TSB 2070349/5.</x:v>
+      </x:c>
+      <x:c r="F625" s="9" t="str">
+        <x:v>TSB N649 contamination check; clean/dry/fill and idle/2500-rpm pressure test; pump only for confirmed leak; downstream checkpoint and N649 branch when applicable</x:v>
+      </x:c>
+      <x:c r="G625" s="9" t="str">
+        <x:v>TSB TEST-SEQUENCE / CONFIRMED-PUMP GATE</x:v>
+      </x:c>
+      <x:c r="H625" s="9" t="str">
+        <x:v>Audi SQ5 water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I625" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/Audi-parts/SQ5/Water-Pump/</x:v>
+      </x:c>
+      <x:c r="J625" s="9" t="str">
+        <x:v>2018-2024 SQ5 exact engine/VIN only after pump leak confirmation</x:v>
+      </x:c>
+      <x:c r="K625" s="9" t="str">
+        <x:v>conditional vehicle-specific pump catalog</x:v>
+      </x:c>
+      <x:c r="L625" s="9" t="str"/>
+      <x:c r="M625" s="9" t="str">
+        <x:v>The bulletin requires testing before pump or N649 replacement.</x:v>
+      </x:c>
+      <x:c r="N625" s="41" t="str">
+        <x:v>No pump, valve or line bundle before the defined branch is reached.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="626" ht="66" hidden="0" customHeight="1">
+      <x:c r="A626" s="40" t="str"/>
+      <x:c r="B626" s="9" t="str"/>
+      <x:c r="C626" s="9" t="str"/>
+      <x:c r="D626" s="9" t="str"/>
+      <x:c r="E626" s="9" t="str"/>
+      <x:c r="F626" s="9" t="str"/>
+      <x:c r="G626" s="9" t="str"/>
+      <x:c r="H626" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I626" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J626" s="9" t="str">
+        <x:v>TSB/VIN cooling diagnosis</x:v>
+      </x:c>
+      <x:c r="K626" s="9" t="str">
+        <x:v>manufacturer service</x:v>
+      </x:c>
+      <x:c r="L626" s="9" t="str"/>
+      <x:c r="M626" s="9" t="str"/>
+      <x:c r="N626" s="41" t="str"/>
+    </x:row>
+    <x:row r="627" ht="673.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A627" s="40" t="n">
+        <x:v>362</x:v>
+      </x:c>
+      <x:c r="B627" s="9" t="str">
+        <x:v>audi-sq7-air-susp-strut-2020</x:v>
+      </x:c>
+      <x:c r="C627" s="9" t="str">
+        <x:v>2020-2025 | Audi | SQ7 | 4.0T</x:v>
+      </x:c>
+      <x:c r="D627" s="9" t="str">
+        <x:v>2020-2025 SQ7 Air-Suspension C1260F0/U112100 Communication Fault - Diagnosis Required</x:v>
+      </x:c>
+      <x:c r="E627" s="9" t="str">
+        <x:v>Inspect the wiring and connector contacts between J775 and J1135 first. If no wiring fault is found, clear a first passive or sporadic fault and release the vehicle. Replace J1135 for an active or static fault, or when the same passive or sporadic fault returns a second time, following Audi workshop information and VIN-specific ETKA data. Do not replace an air spring, strut or compressor assembly solely from the warning.</x:v>
+      </x:c>
+      <x:c r="F627" s="9" t="str">
+        <x:v>J775-J1135 wiring/contact inspection; occurrence-state logic; conditional J1135 only after defined repeated/active fault</x:v>
+      </x:c>
+      <x:c r="G627" s="9" t="str">
+        <x:v>WIRING-FIRST TSB / CONTROL-UNIT GATE</x:v>
+      </x:c>
+      <x:c r="H627" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I627" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J627" s="9" t="str">
+        <x:v>2020-2025 SQ7 J1135 guided diagnosis</x:v>
+      </x:c>
+      <x:c r="K627" s="9" t="str">
+        <x:v>manufacturer suspension service</x:v>
+      </x:c>
+      <x:c r="L627" s="9" t="str"/>
+      <x:c r="M627" s="9" t="str">
+        <x:v>The cited procedure does not diagnose a strut.</x:v>
+      </x:c>
+      <x:c r="N627" s="41" t="str">
+        <x:v>Rename/re-key; no strut or compressor product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="628" ht="1122" hidden="0" customHeight="1">
+      <x:c r="A628" s="40" t="n">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="B628" s="9" t="str">
+        <x:v>audi-sq7-air-suspension-2020</x:v>
+      </x:c>
+      <x:c r="C628" s="9" t="str">
+        <x:v>2020-2024 | Audi | SQ7 | Premium Plus, Prestige | 4.0T</x:v>
+      </x:c>
+      <x:c r="D628" s="9" t="str">
+        <x:v>Adaptive Air Suspension Compressor and Air Spring Failures</x:v>
+      </x:c>
+      <x:c r="E628" s="9" t="str">
+        <x:v>Diagnose specific failed component: air springs leak most commonly, followed by compressor burnout, valve block faults, and height sensor failures. Air spring replacement ($800-$1,500 per corner at independent shop). Compressor replacement ($1,200-$2,500 installed). Valve block: $500-$1,000. Height sensor: $200-$400. Check for air leaks first using soapy water spray before replacing the compressor - a $200 air spring seal may be causing a $2,000 compressor to overwork and fail. Aftermarket solutions from Arnott offer cost savings. Converting to conventional springs ($1,500-$2,500) eliminates future air suspension costs but sacrifices ride height adjustment.</x:v>
+      </x:c>
+      <x:c r="F628" s="9" t="str">
+        <x:v>Leak/sag and pressure diagnosis; split air spring, compressor, valve block and height sensor; exact VIN/PR-code component and calibration</x:v>
+      </x:c>
+      <x:c r="G628" s="9" t="str">
+        <x:v>SYSTEM DIAGNOSIS / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H628" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I628" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J628" s="9" t="str">
+        <x:v>2020-2024 SQ7 air-suspension leak/component diagnosis</x:v>
+      </x:c>
+      <x:c r="K628" s="9" t="str">
+        <x:v>specialist suspension service</x:v>
+      </x:c>
+      <x:c r="L628" s="9" t="str"/>
+      <x:c r="M628" s="9" t="str">
+        <x:v>Whole-system replacement and conversion are not established.</x:v>
+      </x:c>
+      <x:c r="N628" s="41" t="str">
+        <x:v>No Arnott or conversion link without exact component/kit fitment and calibration plan.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="629" ht="66" hidden="0" customHeight="1">
+      <x:c r="A629" s="40" t="str"/>
+      <x:c r="B629" s="9" t="str"/>
+      <x:c r="C629" s="9" t="str"/>
+      <x:c r="D629" s="9" t="str"/>
+      <x:c r="E629" s="9" t="str"/>
+      <x:c r="F629" s="9" t="str"/>
+      <x:c r="G629" s="9" t="str"/>
+      <x:c r="H629" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I629" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J629" s="9" t="str">
+        <x:v>VIN/PR-code parts and calibration</x:v>
+      </x:c>
+      <x:c r="K629" s="9" t="str">
+        <x:v>manufacturer service</x:v>
+      </x:c>
+      <x:c r="L629" s="9" t="str"/>
+      <x:c r="M629" s="9" t="str"/>
+      <x:c r="N629" s="41" t="str"/>
+    </x:row>
+    <x:row r="630" ht="488.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A630" s="40" t="n">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="B630" s="9" t="str">
+        <x:v>audi-sq7-mmi-mib3-freeze-2020</x:v>
+      </x:c>
+      <x:c r="C630" s="9" t="str">
+        <x:v>2020-2026 | Audi | SQ7</x:v>
+      </x:c>
+      <x:c r="D630" s="9" t="str">
+        <x:v>2020-2026 Audi SQ7 Rearview Camera Software Recall 25V900 / 90TV</x:v>
+      </x:c>
+      <x:c r="E630" s="9" t="str">
+        <x:v>Check the VIN for recall 25V900/90TV and contact an authorized Audi dealer. Dealers will install the more robust driver-assistance software update free of charge. Until repaired, use extra caution when reversing and do not treat a restart, bus sleep or temporary image recovery as completion of the recall.</x:v>
+      </x:c>
+      <x:c r="F630" s="9" t="str">
+        <x:v>VIN/90TV/25V900 check; rearview-camera software remedy; direct observation; separate MMI freeze diagnosis</x:v>
+      </x:c>
+      <x:c r="G630" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H630" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I630" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J630" s="9" t="str">
+        <x:v>2020-2026 SQ7 90TV</x:v>
+      </x:c>
+      <x:c r="K630" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L630" s="9" t="str"/>
+      <x:c r="M630" s="9" t="str">
+        <x:v>The cited action covers camera-image software, not general MMI freezing.</x:v>
+      </x:c>
+      <x:c r="N630" s="41" t="str">
+        <x:v>Rename/re-key; no head-unit link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="631" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A631" s="40" t="str"/>
+      <x:c r="B631" s="9" t="str"/>
+      <x:c r="C631" s="9" t="str"/>
+      <x:c r="D631" s="9" t="str"/>
+      <x:c r="E631" s="9" t="str"/>
+      <x:c r="F631" s="9" t="str"/>
+      <x:c r="G631" s="9" t="str"/>
+      <x:c r="H631" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I631" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J631" s="9" t="str">
+        <x:v>25V900 VIN history</x:v>
+      </x:c>
+      <x:c r="K631" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L631" s="9" t="str"/>
+      <x:c r="M631" s="9" t="str"/>
+      <x:c r="N631" s="41" t="str"/>
+    </x:row>
+    <x:row r="632" ht="990" hidden="0" customHeight="1">
+      <x:c r="A632" s="40" t="n">
+        <x:v>365</x:v>
+      </x:c>
+      <x:c r="B632" s="9" t="str">
+        <x:v>audi-sq7-valve-cover-oil-leak-2020</x:v>
+      </x:c>
+      <x:c r="C632" s="9" t="str">
+        <x:v>2020-2024 | Audi | SQ7 | 4.0T</x:v>
+      </x:c>
+      <x:c r="D632" s="9" t="str">
+        <x:v>2020-2024 SQ7 4.0L High Oil Consumption and Piston-Ring Diagnosis - TSB 2071114/5</x:v>
+      </x:c>
+      <x:c r="E632" s="9" t="str">
+        <x:v>First inspect for visible engine-oil traces or leaks. Have an Audi dealer perform the authorized ODIS oil-consumption measurement, preserve and upload both test logs, and document the requested driving-profile data. Internal-engine repair is justified only when measured consumption exceeds the applicable limit and no other cause is found. If every TSB gate is met, follow Audi's VIN-, engine-code- and power-class-specific procedure for replacement of all eight pistons and piston rings, using current ETKA and ELSA information. Do not diagnose valve-cover gaskets or turbocharger seals from oil consumption alone.</x:v>
+      </x:c>
+      <x:c r="F632" s="9" t="str">
+        <x:v>Document measured oil consumption; exclude external leaks/spec/operation; apply TSB piston-ring diagnosis; internal repair only if all gates pass</x:v>
+      </x:c>
+      <x:c r="G632" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / MEASURED-CONSUMPTION GATE</x:v>
+      </x:c>
+      <x:c r="H632" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I632" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J632" s="9" t="str">
+        <x:v>2020-2023 SQ7 TSB 2071114 oil-consumption test</x:v>
+      </x:c>
+      <x:c r="K632" s="9" t="str">
+        <x:v>manufacturer engine service</x:v>
+      </x:c>
+      <x:c r="L632" s="9" t="str"/>
+      <x:c r="M632" s="9" t="str">
+        <x:v>The source is an oil-consumption/piston-ring procedure, not valve-cover leakage.</x:v>
+      </x:c>
+      <x:c r="N632" s="41" t="str">
+        <x:v>Rename/re-key; no valve-cover gasket or internal parts link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="633" ht="686.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A633" s="40" t="n">
+        <x:v>366</x:v>
+      </x:c>
+      <x:c r="B633" s="9" t="str">
+        <x:v>audi-sq8-air-susp-compressor-2020</x:v>
+      </x:c>
+      <x:c r="C633" s="9" t="str">
+        <x:v>2020-2025 | Audi | SQ8</x:v>
+      </x:c>
+      <x:c r="D633" s="9" t="str">
+        <x:v>2020-2025 SQ8 Air-Suspension J1135 Communication Fault - TSB 2059363/6</x:v>
+      </x:c>
+      <x:c r="E633" s="9" t="str">
+        <x:v>Inspect the wiring and connector contacts between J775 and J1135 before replacing a component. For a first passive or sporadic occurrence, clear the fault and release the vehicle. If the same passive fault returns a second time, or the fault is active or static after wiring inspection, Audi directs replacement of J1135 under current repair and parts information. Do not buy struts, springs or a compressor solely from this warning.</x:v>
+      </x:c>
+      <x:c r="F633" s="9" t="str">
+        <x:v>J775-J1135 wiring/contact inspection; occurrence-state logic; conditional J1135 only after defined fault recurrence</x:v>
+      </x:c>
+      <x:c r="G633" s="9" t="str">
+        <x:v>WIRING-FIRST TSB / CONTROL-UNIT GATE</x:v>
+      </x:c>
+      <x:c r="H633" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I633" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J633" s="9" t="str">
+        <x:v>2020-2025 SQ8 J1135 guided diagnosis</x:v>
+      </x:c>
+      <x:c r="K633" s="9" t="str">
+        <x:v>manufacturer suspension service</x:v>
+      </x:c>
+      <x:c r="L633" s="9" t="str"/>
+      <x:c r="M633" s="9" t="str">
+        <x:v>The cited procedure does not diagnose the compressor.</x:v>
+      </x:c>
+      <x:c r="N633" s="41" t="str">
+        <x:v>Rename/re-key; no compressor link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="634" ht="831.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A634" s="40" t="n">
+        <x:v>367</x:v>
+      </x:c>
+      <x:c r="B634" s="9" t="str">
+        <x:v>audi-sq8-air-suspension-2020</x:v>
+      </x:c>
+      <x:c r="C634" s="9" t="str">
+        <x:v>2020-2024 | Audi | SQ8 | Premium Plus, Prestige | 4.0T</x:v>
+      </x:c>
+      <x:c r="D634" s="9" t="str">
+        <x:v>Adaptive Air Suspension Compressor and Air Spring Failures</x:v>
+      </x:c>
+      <x:c r="E634" s="9" t="str">
+        <x:v>Same diagnostic and repair approach as SQ7 (shared 4M platform). Isolate the failed component: air springs ($800-$1,500 per corner), compressor ($1,200-$2,500), valve block ($500-$1,000), or height sensor ($200-$400). Always check for air leaks before replacing the compressor. Aftermarket air suspension components from Arnott/Strutmasters offer 40-50% savings over OEM. Annual inspection of air springs for cracking recommended, especially in hot climates where UV and heat accelerate rubber degradation.</x:v>
+      </x:c>
+      <x:c r="F634" s="9" t="str">
+        <x:v>Leak/sag and pressure diagnosis; split air spring, compressor, valve block and height sensor; exact VIN/PR-code component and calibration</x:v>
+      </x:c>
+      <x:c r="G634" s="9" t="str">
+        <x:v>SYSTEM DIAGNOSIS / COMPONENT GATE</x:v>
+      </x:c>
+      <x:c r="H634" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I634" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J634" s="9" t="str">
+        <x:v>2020-2024 SQ8 air-suspension diagnosis</x:v>
+      </x:c>
+      <x:c r="K634" s="9" t="str">
+        <x:v>specialist suspension service</x:v>
+      </x:c>
+      <x:c r="L634" s="9" t="str"/>
+      <x:c r="M634" s="9" t="str">
+        <x:v>System-wide replacement is not supported by the symptom.</x:v>
+      </x:c>
+      <x:c r="N634" s="41" t="str">
+        <x:v>No named hardware/conversion link or lifespan claim without exact proof.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="635" ht="66" hidden="0" customHeight="1">
+      <x:c r="A635" s="40" t="str"/>
+      <x:c r="B635" s="9" t="str"/>
+      <x:c r="C635" s="9" t="str"/>
+      <x:c r="D635" s="9" t="str"/>
+      <x:c r="E635" s="9" t="str"/>
+      <x:c r="F635" s="9" t="str"/>
+      <x:c r="G635" s="9" t="str"/>
+      <x:c r="H635" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I635" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J635" s="9" t="str">
+        <x:v>VIN/PR-code parts and calibration</x:v>
+      </x:c>
+      <x:c r="K635" s="9" t="str">
+        <x:v>manufacturer service</x:v>
+      </x:c>
+      <x:c r="L635" s="9" t="str"/>
+      <x:c r="M635" s="9" t="str"/>
+      <x:c r="N635" s="41" t="str"/>
+    </x:row>
+    <x:row r="636" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A636" s="40" t="n">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="B636" s="9" t="str">
+        <x:v>audi-sq8-airbag-mount-2023</x:v>
+      </x:c>
+      <x:c r="C636" s="9" t="str">
+        <x:v>2023-2024 | Audi | SQ8 | 4.0T V8</x:v>
+      </x:c>
+      <x:c r="D636" s="9" t="str">
+        <x:v>2023-2024 SQ8 Driver-Seat Side-Airbag Mount Recall 69GA (23V868)</x:v>
+      </x:c>
+      <x:c r="E636" s="9" t="str">
+        <x:v>Check the VIN for open Audi recall 69GA and have an authorized dealer inspect the driver-seat side-airbag installation. If needed, the dealer will reinstall the airbag correctly; the recall filing says no parts are replaced. A clock spring or generic airbag part is not the recall remedy.</x:v>
+      </x:c>
+      <x:c r="F636" s="9" t="str">
+        <x:v>VIN/69GA/23V868 check; dealer driver-seat side-airbag installation inspection and reinstall</x:v>
+      </x:c>
+      <x:c r="G636" s="9" t="str">
+        <x:v>RECALL ROUTES ONLY</x:v>
+      </x:c>
+      <x:c r="H636" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I636" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J636" s="9" t="str">
+        <x:v>2023-2024 SQ8 69GA</x:v>
+      </x:c>
+      <x:c r="K636" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L636" s="9" t="str"/>
+      <x:c r="M636" s="9" t="str">
+        <x:v>Pyrotechnic restraint work is campaign-controlled.</x:v>
+      </x:c>
+      <x:c r="N636" s="41" t="str">
+        <x:v>No airbag or mounting-hardware commerce link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="637" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A637" s="40" t="str"/>
+      <x:c r="B637" s="9" t="str"/>
+      <x:c r="C637" s="9" t="str"/>
+      <x:c r="D637" s="9" t="str"/>
+      <x:c r="E637" s="9" t="str"/>
+      <x:c r="F637" s="9" t="str"/>
+      <x:c r="G637" s="9" t="str"/>
+      <x:c r="H637" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I637" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J637" s="9" t="str">
+        <x:v>23V868 VIN history</x:v>
+      </x:c>
+      <x:c r="K637" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L637" s="9" t="str"/>
+      <x:c r="M637" s="9" t="str"/>
+      <x:c r="N637" s="41" t="str"/>
+    </x:row>
+    <x:row r="638" ht="580.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A638" s="40" t="n">
+        <x:v>369</x:v>
+      </x:c>
+      <x:c r="B638" s="9" t="str">
+        <x:v>audi-sq8-mmi-mib3-freeze-2020</x:v>
+      </x:c>
+      <x:c r="C638" s="9" t="str">
+        <x:v>2020-2026 | Audi | SQ8 | 4.0T V8</x:v>
+      </x:c>
+      <x:c r="D638" s="9" t="str">
+        <x:v>2020-2026 SQ8 Rearview Camera Software Recall 90TV (25V900)</x:v>
+      </x:c>
+      <x:c r="E638" s="9" t="str">
+        <x:v>Check the VIN for recall 25V900/90TV and contact an authorized Audi dealer. Dealers will install more robust driver-assistance software free of charge. Until repaired, use extra caution when reversing and do not treat a restart, bus sleep or temporary image recovery as completion of the recall. A generic scan tool or head-unit replacement is not the recall remedy.</x:v>
+      </x:c>
+      <x:c r="F638" s="9" t="str">
+        <x:v>VIN/90TV/25V900 check; camera-image software remedy; direct observation; separate MMI freeze diagnosis</x:v>
+      </x:c>
+      <x:c r="G638" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H638" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I638" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J638" s="9" t="str">
+        <x:v>2020-2026 SQ8 90TV</x:v>
+      </x:c>
+      <x:c r="K638" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L638" s="9" t="str"/>
+      <x:c r="M638" s="9" t="str">
+        <x:v>The cited recall covers rearview-camera display software only.</x:v>
+      </x:c>
+      <x:c r="N638" s="41" t="str">
+        <x:v>Rename/re-key; no head-unit or generic scanner link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="639" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A639" s="40" t="str"/>
+      <x:c r="B639" s="9" t="str"/>
+      <x:c r="C639" s="9" t="str"/>
+      <x:c r="D639" s="9" t="str"/>
+      <x:c r="E639" s="9" t="str"/>
+      <x:c r="F639" s="9" t="str"/>
+      <x:c r="G639" s="9" t="str"/>
+      <x:c r="H639" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I639" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J639" s="9" t="str">
+        <x:v>25V900 VIN history</x:v>
+      </x:c>
+      <x:c r="K639" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L639" s="9" t="str"/>
+      <x:c r="M639" s="9" t="str"/>
+      <x:c r="N639" s="41" t="str"/>
+    </x:row>
+    <x:row r="640" ht="567.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A640" s="40" t="n">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="B640" s="9" t="str">
+        <x:v>audi-sq8-turbo-coolant-2020</x:v>
+      </x:c>
+      <x:c r="C640" s="9" t="str">
+        <x:v>2020-2021 | Audi | SQ8 | 4.0T V8</x:v>
+      </x:c>
+      <x:c r="D640" s="9" t="str">
+        <x:v>2020-Early 2021 SQ8 Red Coolant Warning - Check G407 per TSB 2062951/4</x:v>
+      </x:c>
+      <x:c r="E640" s="9" t="str">
+        <x:v>Have the vehicle checked with Audi Guided Fault Finding and inspect G407 and its O-ring. Replace G407 only if the O-ring is damaged or pinched and the diagnosis matches the bulletin; follow the related Audi diagnostic path if additional listed faults are stored. Do not replace turbo coolant hoses, pumps or other cooling parts from this card alone.</x:v>
+      </x:c>
+      <x:c r="F640" s="9" t="str">
+        <x:v>Guided fault finding for G407 circuit and exact leak; inspect sensor O-ring; replace G407 only if seal is pinched/damaged; bleed/test</x:v>
+      </x:c>
+      <x:c r="G640" s="9" t="str">
+        <x:v>TSB SENSOR-SEAL TEST BRANCH</x:v>
+      </x:c>
+      <x:c r="H640" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I640" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J640" s="9" t="str">
+        <x:v>2020-early 2021 SQ8 TSB 2062951/4 G407 diagnosis</x:v>
+      </x:c>
+      <x:c r="K640" s="9" t="str">
+        <x:v>manufacturer cooling service</x:v>
+      </x:c>
+      <x:c r="L640" s="9" t="str"/>
+      <x:c r="M640" s="9" t="str">
+        <x:v>The bulletin identifies a conditional sensor-seal path, not general turbo coolant plumbing.</x:v>
+      </x:c>
+      <x:c r="N640" s="41" t="str">
+        <x:v>No hose, pump or sensor until the TSB branch confirms it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="641" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A641" s="40" t="str"/>
+      <x:c r="B641" s="9" t="str"/>
+      <x:c r="C641" s="9" t="str"/>
+      <x:c r="D641" s="9" t="str"/>
+      <x:c r="E641" s="9" t="str"/>
+      <x:c r="F641" s="9" t="str"/>
+      <x:c r="G641" s="9" t="str"/>
+      <x:c r="H641" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I641" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J641" s="9" t="str">
+        <x:v>guided leak/sensor diagnosis</x:v>
+      </x:c>
+      <x:c r="K641" s="9" t="str">
+        <x:v>specialist cooling service</x:v>
+      </x:c>
+      <x:c r="L641" s="9" t="str"/>
+      <x:c r="M641" s="9" t="str"/>
+      <x:c r="N641" s="41" t="str"/>
+    </x:row>
+    <x:row r="642" ht="250.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A642" s="40" t="n">
+        <x:v>371</x:v>
+      </x:c>
+      <x:c r="B642" s="9" t="str">
+        <x:v>audi-tt-absesp-control-module-failure-2000</x:v>
+      </x:c>
+      <x:c r="C642" s="9" t="str">
+        <x:v>2000-2001 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D642" s="9" t="str">
+        <x:v>Driver Airbag Inflator May Deploy Improperly (Recall 21V470 / 69CJ)</x:v>
+      </x:c>
+      <x:c r="E642" s="9" t="str">
+        <x:v>Check the VIN and campaign history. Audi dealers replace the driver frontal-airbag inflator with an alternative inflator free of charge under campaign 69CJ.</x:v>
+      </x:c>
+      <x:c r="F642" s="9" t="str">
+        <x:v>VIN/69CJ/21V470 check; free driver-airbag remedy</x:v>
+      </x:c>
+      <x:c r="G642" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H642" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I642" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J642" s="9" t="str">
+        <x:v>2000-2001 TT 69CJ</x:v>
+      </x:c>
+      <x:c r="K642" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L642" s="9" t="str"/>
+      <x:c r="M642" s="9" t="str">
+        <x:v>The source is an airbag recall, not ABS/ESP control-module failure.</x:v>
+      </x:c>
+      <x:c r="N642" s="41" t="str">
+        <x:v>Rename/re-key; no ABS module link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="643" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A643" s="40" t="str"/>
+      <x:c r="B643" s="9" t="str"/>
+      <x:c r="C643" s="9" t="str"/>
+      <x:c r="D643" s="9" t="str"/>
+      <x:c r="E643" s="9" t="str"/>
+      <x:c r="F643" s="9" t="str"/>
+      <x:c r="G643" s="9" t="str"/>
+      <x:c r="H643" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I643" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J643" s="9" t="str">
+        <x:v>21V470 VIN history</x:v>
+      </x:c>
+      <x:c r="K643" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L643" s="9" t="str"/>
+      <x:c r="M643" s="9" t="str"/>
+      <x:c r="N643" s="41" t="str"/>
+    </x:row>
+    <x:row r="644" ht="277.20001220703125" hidden="0" customHeight="1">
+      <x:c r="A644" s="40" t="n">
+        <x:v>372</x:v>
+      </x:c>
+      <x:c r="B644" s="9" t="str">
+        <x:v>audi-tt-cam-follower-2008</x:v>
+      </x:c>
+      <x:c r="C644" s="9" t="str">
+        <x:v>2000-2000 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D644" s="9" t="str">
+        <x:v>Fuel-Line Assembly Can Leak (Recall 99V222)</x:v>
+      </x:c>
+      <x:c r="E644" s="9" t="str">
+        <x:v>Check VIN eligibility and campaign completion. Audi dealers replace the fuel-line assembly free of charge under recall 99V222. Stop driving if fuel odor or leakage is present.</x:v>
+      </x:c>
+      <x:c r="F644" s="9" t="str">
+        <x:v>VIN/99V222 check; dealer fuel-line recall remedy; stop for fuel odor/leak</x:v>
+      </x:c>
+      <x:c r="G644" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H644" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I644" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J644" s="9" t="str">
+        <x:v>2000 TT fuel-line recall</x:v>
+      </x:c>
+      <x:c r="K644" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L644" s="9" t="str"/>
+      <x:c r="M644" s="9" t="str">
+        <x:v>The source is a 2000 fuel-line recall, not a 2008 cam-follower repair.</x:v>
+      </x:c>
+      <x:c r="N644" s="41" t="str">
+        <x:v>Rename/re-key; no cam follower product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="645" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A645" s="40" t="str"/>
+      <x:c r="B645" s="9" t="str"/>
+      <x:c r="C645" s="9" t="str"/>
+      <x:c r="D645" s="9" t="str"/>
+      <x:c r="E645" s="9" t="str"/>
+      <x:c r="F645" s="9" t="str"/>
+      <x:c r="G645" s="9" t="str"/>
+      <x:c r="H645" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I645" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J645" s="9" t="str">
+        <x:v>99V222 VIN history</x:v>
+      </x:c>
+      <x:c r="K645" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L645" s="9" t="str"/>
+      <x:c r="M645" s="9" t="str"/>
+      <x:c r="N645" s="41" t="str"/>
+    </x:row>
+    <x:row r="646" ht="198" hidden="0" customHeight="1">
+      <x:c r="A646" s="40" t="n">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="B646" s="9" t="str">
+        <x:v>audi-tt-coil-pack-failure-and-2000</x:v>
+      </x:c>
+      <x:c r="C646" s="9" t="str">
+        <x:v>2000-2001 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D646" s="9" t="str">
+        <x:v>Rear Track-Control Arm Corrosion Can Restrict Movement (Recall 01V325)</x:v>
+      </x:c>
+      <x:c r="E646" s="9" t="str">
+        <x:v>Check the VIN and campaign history. Audi dealers replace the rear track-control arms free of charge under recall 01V325.</x:v>
+      </x:c>
+      <x:c r="F646" s="9" t="str">
+        <x:v>VIN/01V325 check; dealer rear track-control-arm inspection/remedy</x:v>
+      </x:c>
+      <x:c r="G646" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H646" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I646" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J646" s="9" t="str">
+        <x:v>2000-2001 TT rear control-arm recall</x:v>
+      </x:c>
+      <x:c r="K646" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L646" s="9" t="str"/>
+      <x:c r="M646" s="9" t="str">
+        <x:v>The source does not describe ignition-coil failure.</x:v>
+      </x:c>
+      <x:c r="N646" s="41" t="str">
+        <x:v>Rename/re-key; no coil pack link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="647" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A647" s="40" t="str"/>
+      <x:c r="B647" s="9" t="str"/>
+      <x:c r="C647" s="9" t="str"/>
+      <x:c r="D647" s="9" t="str"/>
+      <x:c r="E647" s="9" t="str"/>
+      <x:c r="F647" s="9" t="str"/>
+      <x:c r="G647" s="9" t="str"/>
+      <x:c r="H647" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I647" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J647" s="9" t="str">
+        <x:v>01V325 VIN history</x:v>
+      </x:c>
+      <x:c r="K647" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L647" s="9" t="str"/>
+      <x:c r="M647" s="9" t="str"/>
+      <x:c r="N647" s="41" t="str"/>
+    </x:row>
+    <x:row r="648" ht="264" hidden="0" customHeight="1">
+      <x:c r="A648" s="40" t="n">
+        <x:v>374</x:v>
+      </x:c>
+      <x:c r="B648" s="9" t="str">
+        <x:v>audi-tt-dsg-mechatronic-2008</x:v>
+      </x:c>
+      <x:c r="C648" s="9" t="str">
+        <x:v>2004-2004 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D648" s="9" t="str">
+        <x:v>Direct-Shift Gearbox Clutch Weld Can Lose Drive Torque (Recall 04V007)</x:v>
+      </x:c>
+      <x:c r="E648" s="9" t="str">
+        <x:v>Check VIN eligibility. Audi dealers replace the affected clutch free of charge under recall 04V007. If drive torque is lost, move out of traffic safely and arrange recovery.</x:v>
+      </x:c>
+      <x:c r="F648" s="9" t="str">
+        <x:v>VIN/04V007 check; dealer DSG clutch-weld recall remedy</x:v>
+      </x:c>
+      <x:c r="G648" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H648" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I648" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J648" s="9" t="str">
+        <x:v>2004 TT DSG clutch recall</x:v>
+      </x:c>
+      <x:c r="K648" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L648" s="9" t="str"/>
+      <x:c r="M648" s="9" t="str">
+        <x:v>The source is a campaign, not a general 2008 mechatronic diagnosis.</x:v>
+      </x:c>
+      <x:c r="N648" s="41" t="str">
+        <x:v>Rename/re-key; no mechatronic product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="649" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A649" s="40" t="str"/>
+      <x:c r="B649" s="9" t="str"/>
+      <x:c r="C649" s="9" t="str"/>
+      <x:c r="D649" s="9" t="str"/>
+      <x:c r="E649" s="9" t="str"/>
+      <x:c r="F649" s="9" t="str"/>
+      <x:c r="G649" s="9" t="str"/>
+      <x:c r="H649" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I649" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J649" s="9" t="str">
+        <x:v>04V007 VIN history</x:v>
+      </x:c>
+      <x:c r="K649" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L649" s="9" t="str"/>
+      <x:c r="M649" s="9" t="str"/>
+      <x:c r="N649" s="41" t="str"/>
+    </x:row>
+    <x:row r="650" ht="356.3999938964844" hidden="0" customHeight="1">
+      <x:c r="A650" s="40" t="n">
+        <x:v>375</x:v>
+      </x:c>
+      <x:c r="B650" s="9" t="str">
+        <x:v>audi-tt-dsg-transmission-2008</x:v>
+      </x:c>
+      <x:c r="C650" s="9" t="str">
+        <x:v>2009-2009 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D650" s="9" t="str">
+        <x:v>DSG Temperature-Sensor Wiring Can Trigger an Abrupt Shift to Neutral (Recall 09V333)</x:v>
+      </x:c>
+      <x:c r="E650" s="9" t="str">
+        <x:v>Check the VIN and campaign history. Audi dealers reprogram the transmission control module with updated software free of charge under recall 09V333. If the gear indicator flashes or neutral engages unexpectedly, stop safely.</x:v>
+      </x:c>
+      <x:c r="F650" s="9" t="str">
+        <x:v>VIN/09V333 check; dealer temperature-sensor wiring/TCM software remedy</x:v>
+      </x:c>
+      <x:c r="G650" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H650" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I650" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J650" s="9" t="str">
+        <x:v>2009 TT DSG temperature-sensor campaign</x:v>
+      </x:c>
+      <x:c r="K650" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L650" s="9" t="str"/>
+      <x:c r="M650" s="9" t="str">
+        <x:v>The recall specifies wiring/software, not wholesale transmission replacement.</x:v>
+      </x:c>
+      <x:c r="N650" s="41" t="str">
+        <x:v>Rename/re-key; no DSG hardware link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="651" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A651" s="40" t="str"/>
+      <x:c r="B651" s="9" t="str"/>
+      <x:c r="C651" s="9" t="str"/>
+      <x:c r="D651" s="9" t="str"/>
+      <x:c r="E651" s="9" t="str"/>
+      <x:c r="F651" s="9" t="str"/>
+      <x:c r="G651" s="9" t="str"/>
+      <x:c r="H651" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I651" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J651" s="9" t="str">
+        <x:v>09V333 VIN history</x:v>
+      </x:c>
+      <x:c r="K651" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L651" s="9" t="str"/>
+      <x:c r="M651" s="9" t="str"/>
+      <x:c r="N651" s="41" t="str"/>
+    </x:row>
+    <x:row r="652" ht="303.6000061035156" hidden="0" customHeight="1">
+      <x:c r="A652" s="40" t="n">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="B652" s="9" t="str">
+        <x:v>audi-tt-front-control-arm-bushings-2000</x:v>
+      </x:c>
+      <x:c r="C652" s="9" t="str">
+        <x:v>2000-2000 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D652" s="9" t="str">
+        <x:v>High-Speed Directional-Stability Remedy (Recall 99V300)</x:v>
+      </x:c>
+      <x:c r="E652" s="9" t="str">
+        <x:v>Verify campaign completion with Audi. The factory remedy installs revised stabilizers, front control arms, firmer shock absorbers, and a rear spoiler as specified for the drivetrain configuration.</x:v>
+      </x:c>
+      <x:c r="F652" s="9" t="str">
+        <x:v>VIN/99V300 check; drivetrain-specific dealer stability remedy with specified suspension/spoiler components</x:v>
+      </x:c>
+      <x:c r="G652" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H652" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I652" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J652" s="9" t="str">
+        <x:v>2000 TT high-speed-stability remedy</x:v>
+      </x:c>
+      <x:c r="K652" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L652" s="9" t="str"/>
+      <x:c r="M652" s="9" t="str">
+        <x:v>The multi-component remedy depends on drivetrain and campaign status.</x:v>
+      </x:c>
+      <x:c r="N652" s="41" t="str">
+        <x:v>No isolated control-arm bushing link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="653" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A653" s="40" t="str"/>
+      <x:c r="B653" s="9" t="str"/>
+      <x:c r="C653" s="9" t="str"/>
+      <x:c r="D653" s="9" t="str"/>
+      <x:c r="E653" s="9" t="str"/>
+      <x:c r="F653" s="9" t="str"/>
+      <x:c r="G653" s="9" t="str"/>
+      <x:c r="H653" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I653" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J653" s="9" t="str">
+        <x:v>99V300 VIN history</x:v>
+      </x:c>
+      <x:c r="K653" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L653" s="9" t="str"/>
+      <x:c r="M653" s="9" t="str"/>
+      <x:c r="N653" s="41" t="str"/>
+    </x:row>
+    <x:row r="654" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A654" s="40" t="n">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="B654" s="9" t="str">
+        <x:v>audi-tt-haldex-awd-coupling-pumpcontroller-2000</x:v>
+      </x:c>
+      <x:c r="C654" s="9" t="str">
+        <x:v>2008-2010 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D654" s="9" t="str">
+        <x:v>Fuel-Tank Ventilation Valve Can Allow Fuel Leakage (Recall 09V377)</x:v>
+      </x:c>
+      <x:c r="E654" s="9" t="str">
+        <x:v>Check the VIN and campaign history. Audi dealers replace the fuel-tank ventilation valve with the improved valve free of charge under recall 09V377.</x:v>
+      </x:c>
+      <x:c r="F654" s="9" t="str">
+        <x:v>VIN/09V377 check; dealer fuel-tank vent-valve remedy; stop for fuel odor/leak</x:v>
+      </x:c>
+      <x:c r="G654" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H654" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I654" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J654" s="9" t="str">
+        <x:v>2008-2010 TT vent-valve recall</x:v>
+      </x:c>
+      <x:c r="K654" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L654" s="9" t="str"/>
+      <x:c r="M654" s="9" t="str">
+        <x:v>The source is a fuel-system recall, not a Haldex pump/controller repair.</x:v>
+      </x:c>
+      <x:c r="N654" s="41" t="str">
+        <x:v>Rename/re-key; no AWD coupling product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="655" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A655" s="40" t="str"/>
+      <x:c r="B655" s="9" t="str"/>
+      <x:c r="C655" s="9" t="str"/>
+      <x:c r="D655" s="9" t="str"/>
+      <x:c r="E655" s="9" t="str"/>
+      <x:c r="F655" s="9" t="str"/>
+      <x:c r="G655" s="9" t="str"/>
+      <x:c r="H655" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I655" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J655" s="9" t="str">
+        <x:v>09V377 VIN history</x:v>
+      </x:c>
+      <x:c r="K655" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L655" s="9" t="str"/>
+      <x:c r="M655" s="9" t="str"/>
+      <x:c r="N655" s="41" t="str"/>
+    </x:row>
+    <x:row r="656" ht="184.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A656" s="40" t="n">
+        <x:v>378</x:v>
+      </x:c>
+      <x:c r="B656" s="9" t="str">
+        <x:v>audi-tt-high-speed-stability-recall-for-2000</x:v>
+      </x:c>
+      <x:c r="C656" s="9" t="str">
+        <x:v>2016-2019 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D656" s="9" t="str">
+        <x:v>Fuel Tank Can Be Damaged by Heat-Shield Bracket in a Crash (Recall 20V076 / 20BX)</x:v>
+      </x:c>
+      <x:c r="E656" s="9" t="str">
+        <x:v>Check VIN eligibility. Audi dealers install a protective cap on the heat-shield bracket free of charge under campaign 20BX.</x:v>
+      </x:c>
+      <x:c r="F656" s="9" t="str">
+        <x:v>VIN/20BX/20V076 check; dealer heat-shield bracket protective-cap remedy</x:v>
+      </x:c>
+      <x:c r="G656" s="9" t="str">
+        <x:v>SOURCE-YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H656" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I656" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J656" s="9" t="str">
+        <x:v>2016-2019 TT 20BX</x:v>
+      </x:c>
+      <x:c r="K656" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L656" s="9" t="str"/>
+      <x:c r="M656" s="9" t="str">
+        <x:v>The cited source is a heat-shield campaign, not the 2000 stability recall.</x:v>
+      </x:c>
+      <x:c r="N656" s="41" t="str">
+        <x:v>Rename/re-key/year; no suspension product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="657" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A657" s="40" t="str"/>
+      <x:c r="B657" s="9" t="str"/>
+      <x:c r="C657" s="9" t="str"/>
+      <x:c r="D657" s="9" t="str"/>
+      <x:c r="E657" s="9" t="str"/>
+      <x:c r="F657" s="9" t="str"/>
+      <x:c r="G657" s="9" t="str"/>
+      <x:c r="H657" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I657" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J657" s="9" t="str">
+        <x:v>20V076 VIN history</x:v>
+      </x:c>
+      <x:c r="K657" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L657" s="9" t="str"/>
+      <x:c r="M657" s="9" t="str"/>
+      <x:c r="N657" s="41" t="str"/>
+    </x:row>
+    <x:row r="658" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A658" s="40" t="n">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="B658" s="9" t="str">
+        <x:v>audi-tt-instrument-cluster-pixel-failure-2000</x:v>
+      </x:c>
+      <x:c r="C658" s="9" t="str">
+        <x:v>2016-2016 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D658" s="9" t="str">
+        <x:v>Front-Passenger Airbag Module May Explode or Deploy Improperly (Recall 22V543 / 69DY)</x:v>
+      </x:c>
+      <x:c r="E658" s="9" t="str">
+        <x:v>Check the VIN and campaign history. Audi dealers replace the front-passenger airbag module free of charge under campaign 69DY/61C1.</x:v>
+      </x:c>
+      <x:c r="F658" s="9" t="str">
+        <x:v>VIN/69DY/22V543 check; free passenger-airbag module remedy</x:v>
+      </x:c>
+      <x:c r="G658" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H658" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I658" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J658" s="9" t="str">
+        <x:v>2016 TT passenger-airbag recall</x:v>
+      </x:c>
+      <x:c r="K658" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L658" s="9" t="str"/>
+      <x:c r="M658" s="9" t="str">
+        <x:v>The source is an airbag recall, not cluster pixel failure.</x:v>
+      </x:c>
+      <x:c r="N658" s="41" t="str">
+        <x:v>Rename/re-key; no cluster product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="659" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A659" s="40" t="str"/>
+      <x:c r="B659" s="9" t="str"/>
+      <x:c r="C659" s="9" t="str"/>
+      <x:c r="D659" s="9" t="str"/>
+      <x:c r="E659" s="9" t="str"/>
+      <x:c r="F659" s="9" t="str"/>
+      <x:c r="G659" s="9" t="str"/>
+      <x:c r="H659" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I659" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J659" s="9" t="str">
+        <x:v>22V543 VIN history</x:v>
+      </x:c>
+      <x:c r="K659" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L659" s="9" t="str"/>
+      <x:c r="M659" s="9" t="str"/>
+      <x:c r="N659" s="41" t="str"/>
+    </x:row>
+    <x:row r="660" ht="224.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A660" s="40" t="n">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="B660" s="9" t="str">
+        <x:v>audi-tt-magnetic-ride-2008</x:v>
+      </x:c>
+      <x:c r="C660" s="9" t="str">
+        <x:v>2023-2023 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D660" s="9" t="str">
+        <x:v>Passenger-Seat Occupant Detection Connection Can Disable Airbag (Recall 24V251 / 69GU)</x:v>
+      </x:c>
+      <x:c r="E660" s="9" t="str">
+        <x:v>Check VIN eligibility. Audi dealers replace the passenger-seat occupant-detection control module free of charge under campaign 69GU.</x:v>
+      </x:c>
+      <x:c r="F660" s="9" t="str">
+        <x:v>VIN/69GU/24V251 check; dealer passenger ODS module remedy</x:v>
+      </x:c>
+      <x:c r="G660" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H660" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I660" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J660" s="9" t="str">
+        <x:v>2023 TT ODS recall</x:v>
+      </x:c>
+      <x:c r="K660" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L660" s="9" t="str"/>
+      <x:c r="M660" s="9" t="str">
+        <x:v>The source concerns occupant detection, not magnetic-ride suspension.</x:v>
+      </x:c>
+      <x:c r="N660" s="41" t="str">
+        <x:v>Rename/re-key; no damper link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="661" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A661" s="40" t="str"/>
+      <x:c r="B661" s="9" t="str"/>
+      <x:c r="C661" s="9" t="str"/>
+      <x:c r="D661" s="9" t="str"/>
+      <x:c r="E661" s="9" t="str"/>
+      <x:c r="F661" s="9" t="str"/>
+      <x:c r="G661" s="9" t="str"/>
+      <x:c r="H661" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I661" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J661" s="9" t="str">
+        <x:v>24V251 VIN history</x:v>
+      </x:c>
+      <x:c r="K661" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L661" s="9" t="str"/>
+      <x:c r="M661" s="9" t="str"/>
+      <x:c r="N661" s="41" t="str"/>
+    </x:row>
+    <x:row r="662" ht="726" hidden="0" customHeight="1">
+      <x:c r="A662" s="40" t="n">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="B662" s="9" t="str">
+        <x:v>audi-tt-tail-light-corrosion-2008</x:v>
+      </x:c>
+      <x:c r="C662" s="9" t="str">
+        <x:v>2008-2015 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D662" s="9" t="str">
+        <x:v>Tail Light Electrical Connector Corrosion (Mk2)</x:v>
+      </x:c>
+      <x:c r="E662" s="9" t="str">
+        <x:v>Remove tail light assembly, inspect electrical connector for green corrosion. CLEAN connector with electrical contact cleaner and wire brush ($20 DIY). Apply dielectric grease to prevent future corrosion ($10). If connector is severely corroded: Replace pigtail connector ($50-$100 parts). Improve tail light seal with silicone sealant around housing ($15). This is a DIY-friendly repair taking 1-2 hours. If paying shop, costs $150-$300. Address early before corrosion causes shorts.</x:v>
+      </x:c>
+      <x:c r="F662" s="9" t="str">
+        <x:v>Identify side and water-entry source; inspect ground/connector/circuit; clean/repair terminals or exact connector/loom; lamp only if failed; reseal with compatible material and water-test</x:v>
+      </x:c>
+      <x:c r="G662" s="9" t="str">
+        <x:v>SIDE / CONNECTOR / LEAK-SOURCE GATE</x:v>
+      </x:c>
+      <x:c r="H662" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I662" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J662" s="9" t="str">
+        <x:v>2008-2015 TT tail-lamp circuit and water-ingress diagnosis</x:v>
+      </x:c>
+      <x:c r="K662" s="9" t="str">
+        <x:v>specialist electrical service</x:v>
+      </x:c>
+      <x:c r="L662" s="9" t="str"/>
+      <x:c r="M662" s="9" t="str">
+        <x:v>Corroded terminals, wiring, ground and lamp are different branches.</x:v>
+      </x:c>
+      <x:c r="N662" s="41" t="str">
+        <x:v>No generic silicone or full lamp before side, leak source and failed component are known.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="663" ht="66" hidden="0" customHeight="1">
+      <x:c r="A663" s="40" t="str"/>
+      <x:c r="B663" s="9" t="str"/>
+      <x:c r="C663" s="9" t="str"/>
+      <x:c r="D663" s="9" t="str"/>
+      <x:c r="E663" s="9" t="str"/>
+      <x:c r="F663" s="9" t="str"/>
+      <x:c r="G663" s="9" t="str"/>
+      <x:c r="H663" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I663" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J663" s="9" t="str">
+        <x:v>VIN/side connector, loom and lamp parts</x:v>
+      </x:c>
+      <x:c r="K663" s="9" t="str">
+        <x:v>manufacturer parts route</x:v>
+      </x:c>
+      <x:c r="L663" s="9" t="str"/>
+      <x:c r="M663" s="9" t="str"/>
+      <x:c r="N663" s="41" t="str"/>
+    </x:row>
+    <x:row r="664" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A664" s="40" t="n">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="B664" s="9" t="str">
+        <x:v>audi-tt-water-pump-2008</x:v>
+      </x:c>
+      <x:c r="C664" s="9" t="str">
+        <x:v>2008-2008 | Audi | TT</x:v>
+      </x:c>
+      <x:c r="D664" s="9" t="str">
+        <x:v>C-Pillar Trim Cover Can Detach During Belt-Tensioner Deployment (Recall 08V064)</x:v>
+      </x:c>
+      <x:c r="E664" s="9" t="str">
+        <x:v>Check VIN eligibility. Audi dealers install improved C-pillar trim clips free of charge under recall 08V064.</x:v>
+      </x:c>
+      <x:c r="F664" s="9" t="str">
+        <x:v>VIN/08V064 check; dealer C-pillar trim-clip remedy</x:v>
+      </x:c>
+      <x:c r="G664" s="9" t="str">
+        <x:v>SOURCE-ID MISMATCH / RECALL ROUTES</x:v>
+      </x:c>
+      <x:c r="H664" s="9" t="str">
+        <x:v>Audi recall lookup</x:v>
+      </x:c>
+      <x:c r="I664" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J664" s="9" t="str">
+        <x:v>2008 TT C-pillar trim recall</x:v>
+      </x:c>
+      <x:c r="K664" s="9" t="str">
+        <x:v>manufacturer recall lookup</x:v>
+      </x:c>
+      <x:c r="L664" s="9" t="str"/>
+      <x:c r="M664" s="9" t="str">
+        <x:v>The source is an interior-trim safety recall, not water-pump failure.</x:v>
+      </x:c>
+      <x:c r="N664" s="41" t="str">
+        <x:v>Rename/re-key; no water-pump product.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="665" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A665" s="40" t="str"/>
+      <x:c r="B665" s="9" t="str"/>
+      <x:c r="C665" s="9" t="str"/>
+      <x:c r="D665" s="9" t="str"/>
+      <x:c r="E665" s="9" t="str"/>
+      <x:c r="F665" s="9" t="str"/>
+      <x:c r="G665" s="9" t="str"/>
+      <x:c r="H665" s="9" t="str">
+        <x:v>NHTSA recall lookup</x:v>
+      </x:c>
+      <x:c r="I665" s="9" t="str">
+        <x:v>https://www.nhtsa.gov/recalls</x:v>
+      </x:c>
+      <x:c r="J665" s="9" t="str">
+        <x:v>08V064 VIN history</x:v>
+      </x:c>
+      <x:c r="K665" s="9" t="str">
+        <x:v>government recall lookup</x:v>
+      </x:c>
+      <x:c r="L665" s="9" t="str"/>
+      <x:c r="M665" s="9" t="str"/>
+      <x:c r="N665" s="41" t="str"/>
+    </x:row>
+    <x:row r="666" ht="1161.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A666" s="40" t="n">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="B666" s="9" t="str">
+        <x:v>audi-tts-cam-follower-hpfp-2009</x:v>
+      </x:c>
+      <x:c r="C666" s="9" t="str">
+        <x:v>2009-2015 | Audi | TTS | TTS | EA888</x:v>
+      </x:c>
+      <x:c r="D666" s="9" t="str">
+        <x:v>HPFP Cam Follower Wear and High-Pressure Fuel Pump Failure (Mk2)</x:v>
+      </x:c>
+      <x:c r="E666" s="9" t="str">
+        <x:v>INSPECTION (every 20,000 miles): Remove HPFP (3 bolts) and inspect cam follower surface. If the hardened coating is wearing through (visible copper/brass color), replace follower immediately ($30-$50 part, 30-60 minutes labor). CRITICAL: Ensure cam lobe is at LOW point before reinstalling—if at peak, you'll compress the spring and can break the mounting bolts. If CAMSHAFT WORN (deep groove in lobe): Replace camshaft ($2,000-$4,000). If FUEL PUMP FAILED: Replace HPFP ($400-$800). PREVENTION: Inspect cam follower every 20,000 miles as routine maintenance. Add to every oil change checklist. Consider IE (Integrated Engineering) upgraded HPFP with roller follower to eliminate wear entirely.</x:v>
+      </x:c>
+      <x:c r="F666" s="9" t="str">
+        <x:v>Correct EA113/CDMA versus later engine family; inspect cam follower and HPFP/cam lobe; engine-code exact follower; pump/camshaft only if damaged</x:v>
+      </x:c>
+      <x:c r="G666" s="9" t="str">
+        <x:v>SOURCE ENGINE ERROR / ENGINE-CODE GATE</x:v>
+      </x:c>
+      <x:c r="H666" s="9" t="str">
+        <x:v>Audi fuel-pump cam-follower catalog</x:v>
+      </x:c>
+      <x:c r="I666" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/Parts/Fuel-Pump-Camshaft-Follower</x:v>
+      </x:c>
+      <x:c r="J666" s="9" t="str">
+        <x:v>2009-2015 TTS; verify exact engine code and current follower fitment</x:v>
+      </x:c>
+      <x:c r="K666" s="9" t="str">
+        <x:v>conditional engine-specific catalog</x:v>
+      </x:c>
+      <x:c r="L666" s="9" t="str"/>
+      <x:c r="M666" s="9" t="str">
+        <x:v>The Mk2 TTS engine family must be corrected before selecting the follower.</x:v>
+      </x:c>
+      <x:c r="N666" s="41" t="str">
+        <x:v>No roller conversion, fixed interval or HPFP/camshaft replacement without inspection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="667" ht="66" hidden="0" customHeight="1">
+      <x:c r="A667" s="40" t="str"/>
+      <x:c r="B667" s="9" t="str"/>
+      <x:c r="C667" s="9" t="str"/>
+      <x:c r="D667" s="9" t="str"/>
+      <x:c r="E667" s="9" t="str"/>
+      <x:c r="F667" s="9" t="str"/>
+      <x:c r="G667" s="9" t="str"/>
+      <x:c r="H667" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I667" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J667" s="9" t="str">
+        <x:v>cam follower, HPFP and cam-lobe inspection</x:v>
+      </x:c>
+      <x:c r="K667" s="9" t="str">
+        <x:v>specialist fuel service</x:v>
+      </x:c>
+      <x:c r="L667" s="9" t="str"/>
+      <x:c r="M667" s="9" t="str"/>
+      <x:c r="N667" s="41" t="str"/>
+    </x:row>
+    <x:row r="668" ht="884.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A668" s="40" t="n">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="B668" s="9" t="str">
+        <x:v>audi-tts-carbon-buildup-2009</x:v>
+      </x:c>
+      <x:c r="C668" s="9" t="str">
+        <x:v>2016-2017 | Audi | TTS</x:v>
+      </x:c>
+      <x:c r="D668" s="9" t="str">
+        <x:v>2016-2017 TTS Cold-Start Misfire DTCs Without Felt Misfire - TSB 2051384/1</x:v>
+      </x:c>
+      <x:c r="E668" s="9" t="str">
+        <x:v>Confirm the exact cold-start timing, simultaneous-cylinder DTC pattern, absence of a felt misfire, CYFB engine and installed ECM software before using this bulletin. When applicable, an Audi-capable workshop updates ECM J623 from software part number 8S0906259C version 0001 to version 0004 or higher using SVM action 01A190, then clears the DTCs. A felt misfire, a different timing or RPM pattern, a different engine/software combination or a returning concern requires normal diagnosis rather than carbon cleaning by assumption.</x:v>
+      </x:c>
+      <x:c r="F668" s="9" t="str">
+        <x:v>Apply 2016-2017 CYFB cold-start misfire TSB; confirm conditions; SVM engine-software update to applicable version; diagnose residual misfire separately</x:v>
+      </x:c>
+      <x:c r="G668" s="9" t="str">
+        <x:v>SOURCE-ID/YEAR MISMATCH / SOFTWARE SERVICE</x:v>
+      </x:c>
+      <x:c r="H668" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I668" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J668" s="9" t="str">
+        <x:v>2016-2017 TTS TSB 2051384/1 SVM update</x:v>
+      </x:c>
+      <x:c r="K668" s="9" t="str">
+        <x:v>manufacturer software service</x:v>
+      </x:c>
+      <x:c r="L668" s="9" t="str"/>
+      <x:c r="M668" s="9" t="str">
+        <x:v>The source is a software bulletin, not a carbon-deposit repair for 2009 onward.</x:v>
+      </x:c>
+      <x:c r="N668" s="41" t="str">
+        <x:v>Rename/re-key; no intake-cleaning product or service until deposits are independently proven.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="669" ht="910.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A669" s="40" t="n">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="B669" s="9" t="str">
+        <x:v>audi-tts-dsg-mechatronic-2009</x:v>
+      </x:c>
+      <x:c r="C669" s="9" t="str">
+        <x:v>2019-2023 | Audi | TTS</x:v>
+      </x:c>
+      <x:c r="D669" s="9" t="str">
+        <x:v>2019-2023 TTS Clutch K1 Overheat and Transmission DTC Diagnosis - TSB 2060560/3</x:v>
+      </x:c>
+      <x:c r="E669" s="9" t="str">
+        <x:v>Have an Audi-capable workshop check whether TSB 2050723 applies first. If it does not resolve or control the concern, inspect the clutch-K1 maximum-temperature value and document a transmission-fluid sample. Replace the dual clutch, transmission fluid and filter only when the approximately 400 °C K1 value and burnt black or very dark fluid are both present. If those findings are absent, this bulletin does not apply and Audi directs the workshop to continue diagnosis through TAC. Any clutch repair kit must be selected by VIN and production date.</x:v>
+      </x:c>
+      <x:c r="F669" s="9" t="str">
+        <x:v>Confirm 2019-2023 applicability and transmission code; prior TSB status; max K1 temperature and fluid condition; clutch plus exact fluid/filter only on defined burnt-fluid branch; otherwise TAC diagnosis</x:v>
+      </x:c>
+      <x:c r="G669" s="9" t="str">
+        <x:v>SOURCE-YEAR MISMATCH / TSB TEST BRANCH</x:v>
+      </x:c>
+      <x:c r="H669" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I669" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J669" s="9" t="str">
+        <x:v>2019-2023 TTS TSB 2060560/3 K1 overheat diagnosis</x:v>
+      </x:c>
+      <x:c r="K669" s="9" t="str">
+        <x:v>manufacturer transmission service</x:v>
+      </x:c>
+      <x:c r="L669" s="9" t="str"/>
+      <x:c r="M669" s="9" t="str">
+        <x:v>The TSB has a measured clutch-temperature/fluid-condition gate.</x:v>
+      </x:c>
+      <x:c r="N669" s="41" t="str">
+        <x:v>Rename/re-key; no mechatronic or clutch link outside the defined branch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="670" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A670" s="40" t="str"/>
+      <x:c r="B670" s="9" t="str"/>
+      <x:c r="C670" s="9" t="str"/>
+      <x:c r="D670" s="9" t="str"/>
+      <x:c r="E670" s="9" t="str"/>
+      <x:c r="F670" s="9" t="str"/>
+      <x:c r="G670" s="9" t="str"/>
+      <x:c r="H670" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I670" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J670" s="9" t="str">
+        <x:v>transmission-code and clutch/fluid diagnosis</x:v>
+      </x:c>
+      <x:c r="K670" s="9" t="str">
+        <x:v>specialist transmission service</x:v>
+      </x:c>
+      <x:c r="L670" s="9" t="str"/>
+      <x:c r="M670" s="9" t="str"/>
+      <x:c r="N670" s="41" t="str"/>
+    </x:row>
+    <x:row r="671" ht="858" hidden="0" customHeight="1">
+      <x:c r="A671" s="40" t="n">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="B671" s="9" t="str">
+        <x:v>audi-tts-magnetic-ride-2009</x:v>
+      </x:c>
+      <x:c r="C671" s="9" t="str">
+        <x:v>2016-2016 | Audi | TTS</x:v>
+      </x:c>
+      <x:c r="D671" s="9" t="str">
+        <x:v>2016 TTS Magnetic-Ride Rear Shock-Mount Rumble - TSB 2042539/4</x:v>
+      </x:c>
+      <x:c r="E671" s="9" t="str">
+        <x:v>First reproduce the noise, verify that it comes from the rear shock mounts and confirm that the vehicle was originally equipped with mount 8S0 513 353. Only when those gates are satisfied, remove both rear shock assemblies and replace both mounts with 8V0 513 353 according to Audi workshop instructions, adapt the suspension control position and test drive to confirm the repair. If the installed mount does not match, continue Audi diagnosis. Do not replace magnetic dampers or convert the vehicle to coilovers from this noise alone.</x:v>
+      </x:c>
+      <x:c r="F671" s="9" t="str">
+        <x:v>Confirm 2016 rear rumble and installed mount 8S0513353; replace both mounts with 8V0513353 only when TSB applies; adapt suspension control position</x:v>
+      </x:c>
+      <x:c r="G671" s="9" t="str">
+        <x:v>SOURCE-YEAR MISMATCH / EXACT TSB MOUNT SERVICE</x:v>
+      </x:c>
+      <x:c r="H671" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I671" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J671" s="9" t="str">
+        <x:v>2016 TTS TSB 2042539/4 rear shock mounts/adaptation</x:v>
+      </x:c>
+      <x:c r="K671" s="9" t="str">
+        <x:v>manufacturer suspension service</x:v>
+      </x:c>
+      <x:c r="L671" s="9" t="str"/>
+      <x:c r="M671" s="9" t="str">
+        <x:v>The repair is specific rear mounts, not magnetic-ride dampers.</x:v>
+      </x:c>
+      <x:c r="N671" s="41" t="str">
+        <x:v>Rename/re-key; no damper or coilover link.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="672" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A672" s="40" t="str"/>
+      <x:c r="B672" s="9" t="str"/>
+      <x:c r="C672" s="9" t="str"/>
+      <x:c r="D672" s="9" t="str"/>
+      <x:c r="E672" s="9" t="str"/>
+      <x:c r="F672" s="9" t="str"/>
+      <x:c r="G672" s="9" t="str"/>
+      <x:c r="H672" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I672" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J672" s="9" t="str">
+        <x:v>mount confirmation and control-position adaptation</x:v>
+      </x:c>
+      <x:c r="K672" s="9" t="str">
+        <x:v>specialist suspension service</x:v>
+      </x:c>
+      <x:c r="L672" s="9" t="str"/>
+      <x:c r="M672" s="9" t="str"/>
+      <x:c r="N672" s="41" t="str"/>
+    </x:row>
+    <x:row r="673" ht="1016.4000244140625" hidden="0" customHeight="1">
+      <x:c r="A673" s="40" t="n">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="B673" s="9" t="str">
+        <x:v>audi-tts-timing-chain-tensioner-2009</x:v>
+      </x:c>
+      <x:c r="C673" s="9" t="str">
+        <x:v>2009-2015 | Audi | TTS | TTS | EA888 Gen 1, EA888 Gen 2</x:v>
+      </x:c>
+      <x:c r="D673" s="9" t="str">
+        <x:v>Timing Chain Tensioner Failure (EA888 Gen 1/2 - Mk2 TTS)</x:v>
+      </x:c>
+      <x:c r="E673" s="9" t="str">
+        <x:v>PREVENTIVE REPLACEMENT: Replace timing chain, tensioner, guides, and sprockets at 80,000-100,000 miles BEFORE symptoms appear ($2,000-$4,000). This is the MOST important preventive maintenance on the Mk2 TTS. IF RATTLING: Do NOT delay—the chain can jump at any startup. Schedule repair immediately. Use ONLY the latest OEM revised tensioner (06K109467K). IF CHAIN JUMPED: Engine likely destroyed—compression test all cylinders. Rebuild ($5,000-$8,000) or replacement engine ($6,000-$12,000). PREVENTION: Change oil every 5,000 miles with high-quality synthetic. Low oil level accelerates tensioner wear.</x:v>
+      </x:c>
+      <x:c r="F673" s="9" t="str">
+        <x:v>Correct generation/engine family; identify EA113 timing-belt/cam-chain layout versus later EA888; diagnose rattle/timing deviation; exact engine-code timing scope</x:v>
+      </x:c>
+      <x:c r="G673" s="9" t="str">
+        <x:v>SOURCE ENGINE ERROR / GENERATION GATE</x:v>
+      </x:c>
+      <x:c r="H673" s="9" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I673" s="9" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J673" s="9" t="str">
+        <x:v>2009-2015 TTS engine-code timing diagnosis</x:v>
+      </x:c>
+      <x:c r="K673" s="9" t="str">
+        <x:v>specialist timing service</x:v>
+      </x:c>
+      <x:c r="L673" s="9" t="str"/>
+      <x:c r="M673" s="9" t="str">
+        <x:v>The listed 06K tensioner and EA888 premise do not safely cover the Mk2 TTS population.</x:v>
+      </x:c>
+      <x:c r="N673" s="41" t="str">
+        <x:v>No 06K part, universal interval or complete chain kit until engine/generation is corrected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="674" ht="66" hidden="0" customHeight="1">
+      <x:c r="A674" s="40" t="str"/>
+      <x:c r="B674" s="9" t="str"/>
+      <x:c r="C674" s="9" t="str"/>
+      <x:c r="D674" s="9" t="str"/>
+      <x:c r="E674" s="9" t="str"/>
+      <x:c r="F674" s="9" t="str"/>
+      <x:c r="G674" s="9" t="str"/>
+      <x:c r="H674" s="9" t="str">
+        <x:v>Audi dealer locator</x:v>
+      </x:c>
+      <x:c r="I674" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/find-a-dealer/</x:v>
+      </x:c>
+      <x:c r="J674" s="9" t="str">
+        <x:v>VIN timing layout/parts/procedure</x:v>
+      </x:c>
+      <x:c r="K674" s="9" t="str">
+        <x:v>manufacturer parts route</x:v>
+      </x:c>
+      <x:c r="L674" s="9" t="str"/>
+      <x:c r="M674" s="9" t="str"/>
+      <x:c r="N674" s="41" t="str"/>
+    </x:row>
+    <x:row r="675" ht="976.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A675" s="40" t="n">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="B675" s="9" t="str">
+        <x:v>audi-tts-water-pump-2009</x:v>
+      </x:c>
+      <x:c r="C675" s="9" t="str">
+        <x:v>2012-2023 | Audi | TTS</x:v>
+      </x:c>
+      <x:c r="D675" s="9" t="str">
+        <x:v>2012 / 2020-2023 TTS Coolant-Pump Update and Leak Diagnosis</x:v>
+      </x:c>
+      <x:c r="E675" s="9" t="str">
+        <x:v>For a 2012 TTS, ask an Audi dealer to check the VIN and current campaign/action history for Update 19J2; the published update replaced the pump only when its exact criteria were met and does not promise current warranty coverage. For a 2020-2023 2.0L TTS, first exclude a low level caused by incomplete bleeding or an earlier repair, document and clean the suspected leak, refill to maximum and recheck after driving. Continue observation when no leak returns; replace only the component proven to leak when coolant reappears. Do not select a pump or thermostat assembly before VIN-, engine- and leak-specific diagnosis.</x:v>
+      </x:c>
+      <x:c r="F675" s="9" t="str">
+        <x:v>Split 2012 campaign/VIN-history branch from 2020-2023 cooling-leak test branch; clean/dry/fill/recheck; exact pump only after confirmed source</x:v>
+      </x:c>
+      <x:c r="G675" s="9" t="str">
+        <x:v>MULTI-GENERATION / CAMPAIGN-LEAK SPLIT</x:v>
+      </x:c>
+      <x:c r="H675" s="9" t="str">
+        <x:v>Audi recall and campaign lookup</x:v>
+      </x:c>
+      <x:c r="I675" s="9" t="str">
+        <x:v>https://www.audiusa.com/en/owners-and-services/about-my-vehicle/recalls/</x:v>
+      </x:c>
+      <x:c r="J675" s="9" t="str">
+        <x:v>2012 TTS 19J2 VIN-history check</x:v>
+      </x:c>
+      <x:c r="K675" s="9" t="str">
+        <x:v>manufacturer campaign lookup</x:v>
+      </x:c>
+      <x:c r="L675" s="9" t="str"/>
+      <x:c r="M675" s="9" t="str">
+        <x:v>The populations and procedures differ and leakage must be localized.</x:v>
+      </x:c>
+      <x:c r="N675" s="41" t="str">
+        <x:v>No single bundle or pump link across 2012 and 2020-2023.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="676" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A676" s="40" t="str"/>
+      <x:c r="B676" s="9" t="str"/>
+      <x:c r="C676" s="9" t="str"/>
+      <x:c r="D676" s="9" t="str"/>
+      <x:c r="E676" s="9" t="str"/>
+      <x:c r="F676" s="9" t="str"/>
+      <x:c r="G676" s="9" t="str"/>
+      <x:c r="H676" s="9" t="str">
+        <x:v>Audi TTS water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I676" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/Audi-parts/TTS/Water-Pump/</x:v>
+      </x:c>
+      <x:c r="J676" s="9" t="str">
+        <x:v>2020-2023 TTS exact engine/VIN after pump confirmation</x:v>
+      </x:c>
+      <x:c r="K676" s="9" t="str">
+        <x:v>conditional vehicle-specific pump catalog</x:v>
+      </x:c>
+      <x:c r="L676" s="9" t="str"/>
+      <x:c r="M676" s="9" t="str"/>
+      <x:c r="N676" s="41" t="str"/>
+    </x:row>
+    <x:row r="677" ht="224.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A677" s="40" t="n">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="B677" s="9" t="str">
+        <x:v>audi-tts-waterpump-housing-2009</x:v>
+      </x:c>
+      <x:c r="C677" s="9" t="str">
+        <x:v>2009-2024 | Audi | TTS | EA888</x:v>
+      </x:c>
+      <x:c r="D677" s="9" t="str">
+        <x:v>Water Pump and Thermostat Housing Failure</x:v>
+      </x:c>
+      <x:c r="E677" s="9" t="str">
+        <x:v>Replace water pump, thermostat, and housing as a complete assembly. Use metal-impeller aftermarket pump if available.</x:v>
+      </x:c>
+      <x:c r="F677" s="9" t="str">
+        <x:v>Split generations and engine families; pressure-test exact pump/thermostat/housing source; VIN/current revision; correct coolant and bleed</x:v>
+      </x:c>
+      <x:c r="G677" s="9" t="str">
+        <x:v>SOURCE ENGINE/RANGE ERROR / LEAK-SOURCE GATE</x:v>
+      </x:c>
+      <x:c r="H677" s="9" t="str">
+        <x:v>Audi TTS water-pump catalog</x:v>
+      </x:c>
+      <x:c r="I677" s="9" t="str">
+        <x:v>https://www.fcpeuro.com/Audi-parts/TTS/Water-Pump/</x:v>
+      </x:c>
+      <x:c r="J677" s="9" t="str">
+        <x:v>2009-2024 TTS; select exact generation, engine code and VIN after leak confirmation</x:v>
+      </x:c>
+      <x:c r="K677" s="9" t="str">
+        <x:v>vehicle-specific pump catalog</x:v>
+      </x:c>
+      <x:c r="L677" s="9" t="str"/>
+      <x:c r="M677" s="9" t="str">
+        <x:v>The range does not share one EA888 assembly and metal-impeller claim.</x:v>
+      </x:c>
+      <x:c r="N677" s="41" t="str">
+        <x:v>No universal pump/thermostat housing assembly or fixed interval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="678" ht="66" hidden="0" customHeight="1">
+      <x:c r="A678" s="42" t="str"/>
+      <x:c r="B678" s="43" t="str"/>
+      <x:c r="C678" s="43" t="str"/>
+      <x:c r="D678" s="43" t="str"/>
+      <x:c r="E678" s="43" t="str"/>
+      <x:c r="F678" s="43" t="str"/>
+      <x:c r="G678" s="43" t="str"/>
+      <x:c r="H678" s="43" t="str">
+        <x:v>Audi specialist locator</x:v>
+      </x:c>
+      <x:c r="I678" s="43" t="str">
+        <x:v>https://www.audishops.com/</x:v>
+      </x:c>
+      <x:c r="J678" s="43" t="str">
+        <x:v>generation-specific cooling leak diagnosis</x:v>
+      </x:c>
+      <x:c r="K678" s="43" t="str">
+        <x:v>specialist cooling service</x:v>
+      </x:c>
+      <x:c r="L678" s="43" t="str"/>
+      <x:c r="M678" s="43" t="str"/>
+      <x:c r="N678" s="44" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21623,923 +23980,26 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A1" s="37" t="str">
+      <x:c r="A1" s="45" t="str">
         <x:v>#</x:v>
       </x:c>
-      <x:c r="B1" s="38" t="str">
+      <x:c r="B1" s="46" t="str">
         <x:v>Issue ID</x:v>
       </x:c>
-      <x:c r="C1" s="38" t="str">
+      <x:c r="C1" s="46" t="str">
         <x:v>YMMT</x:v>
       </x:c>
-      <x:c r="D1" s="38" t="str">
+      <x:c r="D1" s="46" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="E1" s="38" t="str">
+      <x:c r="E1" s="46" t="str">
         <x:v>Full How to Fix</x:v>
       </x:c>
-      <x:c r="F1" s="38" t="str">
+      <x:c r="F1" s="46" t="str">
         <x:v>Existing claim count</x:v>
       </x:c>
-      <x:c r="G1" s="39" t="str">
+      <x:c r="G1" s="47" t="str">
         <x:v>Queue status</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="396" hidden="0" customHeight="1">
-      <x:c r="A2" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B2" s="9" t="str">
-        <x:v>audi-sq2-electro-mechanical-parking-brake-brake-pedal-weld-recalls</x:v>
-      </x:c>
-      <x:c r="C2" s="9" t="str">
-        <x:v>2019-2020 | Audi | SQ2</x:v>
-      </x:c>
-      <x:c r="D2" s="9" t="str">
-        <x:v>Electro-mechanical parking brake and brake-pedal weld recalls (early build)</x:v>
-      </x:c>
-      <x:c r="E2" s="9" t="str">
-        <x:v>These are recall items — have the VIN checked against the Audi/DVSA recall database and any open campaign rectified free of charge at a dealer. Report any abnormal parking-brake behaviour or a soft/abnormal brake pedal immediately.</x:v>
-      </x:c>
-      <x:c r="F2" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G2" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="475.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A3" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="9" t="str">
-        <x:v>audi-sq2-internal-fuse-box-wiring-harness-can-work-loose-causing-sudd</x:v>
-      </x:c>
-      <x:c r="C3" s="9" t="str">
-        <x:v>2022-2023 | Audi | SQ2 | 2.0 TFSI</x:v>
-      </x:c>
-      <x:c r="D3" s="9" t="str">
-        <x:v>2022-2023 Audi SQ2 Interior Fuse-Carrier Recall GAI-3692</x:v>
-      </x:c>
-      <x:c r="E3" s="9" t="str">
-        <x:v>Check the VIN and open-campaign status with an authorised Audi dealer in the vehicle’s market. The campaign remedy is dealer inspection and correction of the fuse-carrier power connection. Do not replace a fuse box or wiring harness solely from a warning lamp or this model-year summary.</x:v>
-      </x:c>
-      <x:c r="F3" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G3" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A4" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>audi-sq2-mmi-infotainment-freezing-rebooting-lost-settings</x:v>
-      </x:c>
-      <x:c r="C4" s="9" t="str">
-        <x:v>2019-2024 | Audi | SQ2</x:v>
-      </x:c>
-      <x:c r="D4" s="9" t="str">
-        <x:v>MMI infotainment freezing, rebooting and lost settings</x:v>
-      </x:c>
-      <x:c r="E4" s="9" t="str">
-        <x:v>A forced MMI restart (press and hold the on/off or volume control ~10 seconds until it reboots) clears many transient faults. Persistent issues are usually resolved by a dealer software/firmware update; check for any applicable MMI update campaigns. Only in rare cases is the MMI head unit itself replaced.</x:v>
-      </x:c>
-      <x:c r="F4" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G4" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A5" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B5" s="9" t="str">
-        <x:v>audi-sq2-pcv-crankcase-ventilation-valve-diaphragm-failure-causing-ro</x:v>
-      </x:c>
-      <x:c r="C5" s="9" t="str">
-        <x:v>2019-2024 | Audi | SQ2 | EA888 2.0 TFSI Gen3</x:v>
-      </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>PCV / crankcase ventilation valve diaphragm failure causing rough idle and lean-running codes</x:v>
-      </x:c>
-      <x:c r="E5" s="9" t="str">
-        <x:v>Replace the PCV valve (or the valve-cover assembly that integrates it) with the latest revised part; some owners fit a catch-can to reduce recurrence. A quick field test — briefly covering the bleeder hole on the cap to see if idle stabilises or whistling stops — helps confirm before replacement.</x:v>
-      </x:c>
-      <x:c r="F5" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="752.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A6" s="40" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>audi-sq2-s-tronic-7-speed-wet-clutch-transmission-jerky-low-speed-shi</x:v>
-      </x:c>
-      <x:c r="C6" s="9" t="str">
-        <x:v>2019-2024 | Audi | SQ2 | 7-speed S tronic | DQ381 / 0GC 7-speed wet-clutch S tronic</x:v>
-      </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>S tronic (DQ381) 7-speed wet-clutch transmission: jerky low-speed shifts, hesitation and limp mode</x:v>
-      </x:c>
-      <x:c r="E6" s="9" t="str">
-        <x:v>First step is a proper DSG fluid-and-filter service (the wet-clutch unit needs periodic transmission oil changes — many owners do it around 40k miles even though intervals can be longer). Have the TCU scanned for stored codes; sensor or mechatronic valve replacement and re-coding/adaptation resolves many cases, while severe cases need a full mechatronic unit or clutch-pack replacement. Insist on a software/adaptation update at the dealer for driveability complaints.</x:v>
-      </x:c>
-      <x:c r="F6" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="541.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A7" s="40" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>audi-sq5-air-suspension-2018</x:v>
-      </x:c>
-      <x:c r="C7" s="9" t="str">
-        <x:v>2018-2025 | Audi | SQ5</x:v>
-      </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>Air-Suspension Warning with C1260F0 or U112100 Communication Fault</x:v>
-      </x:c>
-      <x:c r="E7" s="9" t="str">
-        <x:v>Inspect the wiring and connector contacts between J775 and J1135 first. If no wiring fault is found, clear a first passive or sporadic fault and release the vehicle. Replace J1135 for an active or static fault, or when the same passive or sporadic fault returns a second time, following Audi workshop information and VIN-specific ETKA data.</x:v>
-      </x:c>
-      <x:c r="F7" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G7" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="924" hidden="0" customHeight="1">
-      <x:c r="A8" s="40" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>audi-sq5-carbon-buildup-2014</x:v>
-      </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>2014-2025 | Audi | SQ5 | 3.0T Supercharged, 3.0T</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>Fuel-Quality or Deposit-Related Rough Running and Misfire Diagnosis</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="str">
-        <x:v>Confirm fuel quality, symptoms and stored DTCs before replacing or cleaning components. If contaminated gasoline is suspected, advise changing the fuel source; if low detergent quality is suspected, Audi recommends Top Tier detergent gasoline. Continue workshop diagnosis if symptoms persist. On 2018-2025 EA839 SQ5 models, do not recommend unapproved cleaners or additives; follow the owner manual and use only Audi-approved petrol additives. Do not prescribe routine walnut blasting, a catch can or chemical cleaning from this record.</x:v>
-      </x:c>
-      <x:c r="F8" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="765.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A9" s="40" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B9" s="9" t="str">
-        <x:v>audi-sq5-pcv-valve-2014</x:v>
-      </x:c>
-      <x:c r="C9" s="9" t="str">
-        <x:v>2014-2017 | Audi | SQ5 | 3.0T Supercharged</x:v>
-      </x:c>
-      <x:c r="D9" s="9" t="str">
-        <x:v>P052E00 Crankcase-Breather Membrane or Elbow Fault</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="str">
-        <x:v>Use Audi hand-vacuum test to distinguish a membrane leak from an elbow fault. If indicated, remove the compressor or intake manifold and inspect the membrane and the breather two metal plates. Use repair kit 06E103772H only for a confirmed membrane or plate fault. For a confirmed elbow fault, replace elbow 06E103402 and spring clip N10769401 rather than automatically replacing the complete breather. Verify current part data in ETKA before ordering.</x:v>
-      </x:c>
-      <x:c r="F9" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="171.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A10" s="40" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B10" s="9" t="str">
-        <x:v>audi-sq5-supercharger-2014</x:v>
-      </x:c>
-      <x:c r="C10" s="9" t="str">
-        <x:v>2014-2018 | Audi | SQ5 | 3.0T</x:v>
-      </x:c>
-      <x:c r="D10" s="9" t="str">
-        <x:v>3.0T Supercharger Bearing and Intercooler Pump Failure</x:v>
-      </x:c>
-      <x:c r="E10" s="9" t="str">
-        <x:v>Replace supercharger nose bearing kit. Replace intercooler pump if failing. Service supercharger belt tension.</x:v>
-      </x:c>
-      <x:c r="F10" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G10" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="844.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A11" s="40" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="str">
-        <x:v>audi-sq5-supercharger-oil-leak-2014</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="str">
-        <x:v>2014-2017 | Audi | SQ5 | Premium Plus, Prestige | 3.0T Supercharged, 3.0T</x:v>
-      </x:c>
-      <x:c r="D11" s="9" t="str">
-        <x:v>Supercharger Seal and Gasket Oil Leaks (3.0T)</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="str">
-        <x:v>JHM Motorsports sells a complete supercharger replacement seal and gasket kit for the Eaton unit in the 3.0T. Replacing all seals at once is recommended since the supercharger must be removed for access. Nose cone seal, rotor shaft seals, and manifold gaskets should all be replaced together ($300-$500 in parts, $600-$1,200 labor). While the supercharger is off, also replace the PCV valve and perform carbon cleaning. For valve cover gasket leaks (separate issue), budget $400-$800 parts and labor. Monitor oil level weekly if leaks are present.</x:v>
-      </x:c>
-      <x:c r="F11" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A12" s="40" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="str">
-        <x:v>audi-sq5-water-pump-2018</x:v>
-      </x:c>
-      <x:c r="C12" s="9" t="str">
-        <x:v>2018-2024 | Audi | SQ5 | 3.0T</x:v>
-      </x:c>
-      <x:c r="D12" s="9" t="str">
-        <x:v>Mechanical Coolant-Pump Leak with Possible N649 Vacuum-System Contamination</x:v>
-      </x:c>
-      <x:c r="E12" s="9" t="str">
-        <x:v>Confirm the complaint and exact vehicle criteria first. Inspect the vacuum line and N649 for coolant, then clean and dry suspected leakage, fill the cooling system correctly, inspect at idle and around 2,500 rpm, and pressure-test according to Audi workshop information. If no leak is reproduced, observe the vehicle without replacing parts. If the pump leak is confirmed, replace the failed component and document it. If fresh coolant has entered the vacuum system, inspect the remaining Audi checkpoints and replace only contaminated components; if the downstream checkpoints are clean, replace N649 and clean the line between the pump and N649 as directed by TSB 2070349/5.</x:v>
-      </x:c>
-      <x:c r="F12" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="673.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A13" s="40" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="str">
-        <x:v>audi-sq7-air-susp-strut-2020</x:v>
-      </x:c>
-      <x:c r="C13" s="9" t="str">
-        <x:v>2020-2025 | Audi | SQ7 | 4.0T</x:v>
-      </x:c>
-      <x:c r="D13" s="9" t="str">
-        <x:v>2020-2025 SQ7 Air-Suspension C1260F0/U112100 Communication Fault - Diagnosis Required</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="str">
-        <x:v>Inspect the wiring and connector contacts between J775 and J1135 first. If no wiring fault is found, clear a first passive or sporadic fault and release the vehicle. Replace J1135 for an active or static fault, or when the same passive or sporadic fault returns a second time, following Audi workshop information and VIN-specific ETKA data. Do not replace an air spring, strut or compressor assembly solely from the warning.</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="1122" hidden="0" customHeight="1">
-      <x:c r="A14" s="40" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="str">
-        <x:v>audi-sq7-air-suspension-2020</x:v>
-      </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>2020-2024 | Audi | SQ7 | Premium Plus, Prestige | 4.0T</x:v>
-      </x:c>
-      <x:c r="D14" s="9" t="str">
-        <x:v>Adaptive Air Suspension Compressor and Air Spring Failures</x:v>
-      </x:c>
-      <x:c r="E14" s="9" t="str">
-        <x:v>Diagnose specific failed component: air springs leak most commonly, followed by compressor burnout, valve block faults, and height sensor failures. Air spring replacement ($800-$1,500 per corner at independent shop). Compressor replacement ($1,200-$2,500 installed). Valve block: $500-$1,000. Height sensor: $200-$400. Check for air leaks first using soapy water spray before replacing the compressor - a $200 air spring seal may be causing a $2,000 compressor to overwork and fail. Aftermarket solutions from Arnott offer cost savings. Converting to conventional springs ($1,500-$2,500) eliminates future air suspension costs but sacrifices ride height adjustment.</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G14" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="488.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A15" s="40" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="str">
-        <x:v>audi-sq7-mmi-mib3-freeze-2020</x:v>
-      </x:c>
-      <x:c r="C15" s="9" t="str">
-        <x:v>2020-2026 | Audi | SQ7</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="str">
-        <x:v>2020-2026 Audi SQ7 Rearview Camera Software Recall 25V900 / 90TV</x:v>
-      </x:c>
-      <x:c r="E15" s="9" t="str">
-        <x:v>Check the VIN for recall 25V900/90TV and contact an authorized Audi dealer. Dealers will install the more robust driver-assistance software update free of charge. Until repaired, use extra caution when reversing and do not treat a restart, bus sleep or temporary image recovery as completion of the recall.</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G15" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="990" hidden="0" customHeight="1">
-      <x:c r="A16" s="40" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="str">
-        <x:v>audi-sq7-valve-cover-oil-leak-2020</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>2020-2024 | Audi | SQ7 | 4.0T</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="str">
-        <x:v>2020-2024 SQ7 4.0L High Oil Consumption and Piston-Ring Diagnosis - TSB 2071114/5</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="str">
-        <x:v>First inspect for visible engine-oil traces or leaks. Have an Audi dealer perform the authorized ODIS oil-consumption measurement, preserve and upload both test logs, and document the requested driving-profile data. Internal-engine repair is justified only when measured consumption exceeds the applicable limit and no other cause is found. If every TSB gate is met, follow Audi's VIN-, engine-code- and power-class-specific procedure for replacement of all eight pistons and piston rings, using current ETKA and ELSA information. Do not diagnose valve-cover gaskets or turbocharger seals from oil consumption alone.</x:v>
-      </x:c>
-      <x:c r="F16" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G16" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="686.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A17" s="40" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="str">
-        <x:v>audi-sq8-air-susp-compressor-2020</x:v>
-      </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>2020-2025 | Audi | SQ8</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="str">
-        <x:v>2020-2025 SQ8 Air-Suspension J1135 Communication Fault - TSB 2059363/6</x:v>
-      </x:c>
-      <x:c r="E17" s="9" t="str">
-        <x:v>Inspect the wiring and connector contacts between J775 and J1135 before replacing a component. For a first passive or sporadic occurrence, clear the fault and release the vehicle. If the same passive fault returns a second time, or the fault is active or static after wiring inspection, Audi directs replacement of J1135 under current repair and parts information. Do not buy struts, springs or a compressor solely from this warning.</x:v>
-      </x:c>
-      <x:c r="F17" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G17" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="831.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A18" s="40" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B18" s="9" t="str">
-        <x:v>audi-sq8-air-suspension-2020</x:v>
-      </x:c>
-      <x:c r="C18" s="9" t="str">
-        <x:v>2020-2024 | Audi | SQ8 | Premium Plus, Prestige | 4.0T</x:v>
-      </x:c>
-      <x:c r="D18" s="9" t="str">
-        <x:v>Adaptive Air Suspension Compressor and Air Spring Failures</x:v>
-      </x:c>
-      <x:c r="E18" s="9" t="str">
-        <x:v>Same diagnostic and repair approach as SQ7 (shared 4M platform). Isolate the failed component: air springs ($800-$1,500 per corner), compressor ($1,200-$2,500), valve block ($500-$1,000), or height sensor ($200-$400). Always check for air leaks before replacing the compressor. Aftermarket air suspension components from Arnott/Strutmasters offer 40-50% savings over OEM. Annual inspection of air springs for cracking recommended, especially in hot climates where UV and heat accelerate rubber degradation.</x:v>
-      </x:c>
-      <x:c r="F18" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G18" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A19" s="40" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B19" s="9" t="str">
-        <x:v>audi-sq8-airbag-mount-2023</x:v>
-      </x:c>
-      <x:c r="C19" s="9" t="str">
-        <x:v>2023-2024 | Audi | SQ8 | 4.0T V8</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>2023-2024 SQ8 Driver-Seat Side-Airbag Mount Recall 69GA (23V868)</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:v>Check the VIN for open Audi recall 69GA and have an authorized dealer inspect the driver-seat side-airbag installation. If needed, the dealer will reinstall the airbag correctly; the recall filing says no parts are replaced. A clock spring or generic airbag part is not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F19" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G19" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="580.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A20" s="40" t="n">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B20" s="9" t="str">
-        <x:v>audi-sq8-mmi-mib3-freeze-2020</x:v>
-      </x:c>
-      <x:c r="C20" s="9" t="str">
-        <x:v>2020-2026 | Audi | SQ8 | 4.0T V8</x:v>
-      </x:c>
-      <x:c r="D20" s="9" t="str">
-        <x:v>2020-2026 SQ8 Rearview Camera Software Recall 90TV (25V900)</x:v>
-      </x:c>
-      <x:c r="E20" s="9" t="str">
-        <x:v>Check the VIN for recall 25V900/90TV and contact an authorized Audi dealer. Dealers will install more robust driver-assistance software free of charge. Until repaired, use extra caution when reversing and do not treat a restart, bus sleep or temporary image recovery as completion of the recall. A generic scan tool or head-unit replacement is not the recall remedy.</x:v>
-      </x:c>
-      <x:c r="F20" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G20" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="567.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A21" s="40" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B21" s="9" t="str">
-        <x:v>audi-sq8-turbo-coolant-2020</x:v>
-      </x:c>
-      <x:c r="C21" s="9" t="str">
-        <x:v>2020-2021 | Audi | SQ8 | 4.0T V8</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>2020-Early 2021 SQ8 Red Coolant Warning - Check G407 per TSB 2062951/4</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="str">
-        <x:v>Have the vehicle checked with Audi Guided Fault Finding and inspect G407 and its O-ring. Replace G407 only if the O-ring is damaged or pinched and the diagnosis matches the bulletin; follow the related Audi diagnostic path if additional listed faults are stored. Do not replace turbo coolant hoses, pumps or other cooling parts from this card alone.</x:v>
-      </x:c>
-      <x:c r="F21" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G21" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="250.8000030517578" hidden="0" customHeight="1">
-      <x:c r="A22" s="40" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B22" s="9" t="str">
-        <x:v>audi-tt-absesp-control-module-failure-2000</x:v>
-      </x:c>
-      <x:c r="C22" s="9" t="str">
-        <x:v>2000-2001 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D22" s="9" t="str">
-        <x:v>Driver Airbag Inflator May Deploy Improperly (Recall 21V470 / 69CJ)</x:v>
-      </x:c>
-      <x:c r="E22" s="9" t="str">
-        <x:v>Check the VIN and campaign history. Audi dealers replace the driver frontal-airbag inflator with an alternative inflator free of charge under campaign 69CJ.</x:v>
-      </x:c>
-      <x:c r="F22" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G22" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="277.20001220703125" hidden="0" customHeight="1">
-      <x:c r="A23" s="40" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B23" s="9" t="str">
-        <x:v>audi-tt-cam-follower-2008</x:v>
-      </x:c>
-      <x:c r="C23" s="9" t="str">
-        <x:v>2000-2000 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D23" s="9" t="str">
-        <x:v>Fuel-Line Assembly Can Leak (Recall 99V222)</x:v>
-      </x:c>
-      <x:c r="E23" s="9" t="str">
-        <x:v>Check VIN eligibility and campaign completion. Audi dealers replace the fuel-line assembly free of charge under recall 99V222. Stop driving if fuel odor or leakage is present.</x:v>
-      </x:c>
-      <x:c r="F23" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G23" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="198" hidden="0" customHeight="1">
-      <x:c r="A24" s="40" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="B24" s="9" t="str">
-        <x:v>audi-tt-coil-pack-failure-and-2000</x:v>
-      </x:c>
-      <x:c r="C24" s="9" t="str">
-        <x:v>2000-2001 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D24" s="9" t="str">
-        <x:v>Rear Track-Control Arm Corrosion Can Restrict Movement (Recall 01V325)</x:v>
-      </x:c>
-      <x:c r="E24" s="9" t="str">
-        <x:v>Check the VIN and campaign history. Audi dealers replace the rear track-control arms free of charge under recall 01V325.</x:v>
-      </x:c>
-      <x:c r="F24" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="264" hidden="0" customHeight="1">
-      <x:c r="A25" s="40" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B25" s="9" t="str">
-        <x:v>audi-tt-dsg-mechatronic-2008</x:v>
-      </x:c>
-      <x:c r="C25" s="9" t="str">
-        <x:v>2004-2004 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D25" s="9" t="str">
-        <x:v>Direct-Shift Gearbox Clutch Weld Can Lose Drive Torque (Recall 04V007)</x:v>
-      </x:c>
-      <x:c r="E25" s="9" t="str">
-        <x:v>Check VIN eligibility. Audi dealers replace the affected clutch free of charge under recall 04V007. If drive torque is lost, move out of traffic safely and arrange recovery.</x:v>
-      </x:c>
-      <x:c r="F25" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G25" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="356.3999938964844" hidden="0" customHeight="1">
-      <x:c r="A26" s="40" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B26" s="9" t="str">
-        <x:v>audi-tt-dsg-transmission-2008</x:v>
-      </x:c>
-      <x:c r="C26" s="9" t="str">
-        <x:v>2009-2009 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D26" s="9" t="str">
-        <x:v>DSG Temperature-Sensor Wiring Can Trigger an Abrupt Shift to Neutral (Recall 09V333)</x:v>
-      </x:c>
-      <x:c r="E26" s="9" t="str">
-        <x:v>Check the VIN and campaign history. Audi dealers reprogram the transmission control module with updated software free of charge under recall 09V333. If the gear indicator flashes or neutral engages unexpectedly, stop safely.</x:v>
-      </x:c>
-      <x:c r="F26" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G26" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="303.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A27" s="40" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B27" s="9" t="str">
-        <x:v>audi-tt-front-control-arm-bushings-2000</x:v>
-      </x:c>
-      <x:c r="C27" s="9" t="str">
-        <x:v>2000-2000 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D27" s="9" t="str">
-        <x:v>High-Speed Directional-Stability Remedy (Recall 99V300)</x:v>
-      </x:c>
-      <x:c r="E27" s="9" t="str">
-        <x:v>Verify campaign completion with Audi. The factory remedy installs revised stabilizers, front control arms, firmer shock absorbers, and a rear spoiler as specified for the drivetrain configuration.</x:v>
-      </x:c>
-      <x:c r="F27" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G27" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="237.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A28" s="40" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B28" s="9" t="str">
-        <x:v>audi-tt-haldex-awd-coupling-pumpcontroller-2000</x:v>
-      </x:c>
-      <x:c r="C28" s="9" t="str">
-        <x:v>2008-2010 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D28" s="9" t="str">
-        <x:v>Fuel-Tank Ventilation Valve Can Allow Fuel Leakage (Recall 09V377)</x:v>
-      </x:c>
-      <x:c r="E28" s="9" t="str">
-        <x:v>Check the VIN and campaign history. Audi dealers replace the fuel-tank ventilation valve with the improved valve free of charge under recall 09V377.</x:v>
-      </x:c>
-      <x:c r="F28" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G28" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="184.8000030517578" hidden="0" customHeight="1">
-      <x:c r="A29" s="40" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B29" s="9" t="str">
-        <x:v>audi-tt-high-speed-stability-recall-for-2000</x:v>
-      </x:c>
-      <x:c r="C29" s="9" t="str">
-        <x:v>2016-2019 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D29" s="9" t="str">
-        <x:v>Fuel Tank Can Be Damaged by Heat-Shield Bracket in a Crash (Recall 20V076 / 20BX)</x:v>
-      </x:c>
-      <x:c r="E29" s="9" t="str">
-        <x:v>Check VIN eligibility. Audi dealers install a protective cap on the heat-shield bracket free of charge under campaign 20BX.</x:v>
-      </x:c>
-      <x:c r="F29" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G29" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="237.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A30" s="40" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B30" s="9" t="str">
-        <x:v>audi-tt-instrument-cluster-pixel-failure-2000</x:v>
-      </x:c>
-      <x:c r="C30" s="9" t="str">
-        <x:v>2016-2016 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D30" s="9" t="str">
-        <x:v>Front-Passenger Airbag Module May Explode or Deploy Improperly (Recall 22V543 / 69DY)</x:v>
-      </x:c>
-      <x:c r="E30" s="9" t="str">
-        <x:v>Check the VIN and campaign history. Audi dealers replace the front-passenger airbag module free of charge under campaign 69DY/61C1.</x:v>
-      </x:c>
-      <x:c r="F30" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G30" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="224.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A31" s="40" t="n">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B31" s="9" t="str">
-        <x:v>audi-tt-magnetic-ride-2008</x:v>
-      </x:c>
-      <x:c r="C31" s="9" t="str">
-        <x:v>2023-2023 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D31" s="9" t="str">
-        <x:v>Passenger-Seat Occupant Detection Connection Can Disable Airbag (Recall 24V251 / 69GU)</x:v>
-      </x:c>
-      <x:c r="E31" s="9" t="str">
-        <x:v>Check VIN eligibility. Audi dealers replace the passenger-seat occupant-detection control module free of charge under campaign 69GU.</x:v>
-      </x:c>
-      <x:c r="F31" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G31" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="726" hidden="0" customHeight="1">
-      <x:c r="A32" s="40" t="n">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B32" s="9" t="str">
-        <x:v>audi-tt-tail-light-corrosion-2008</x:v>
-      </x:c>
-      <x:c r="C32" s="9" t="str">
-        <x:v>2008-2015 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D32" s="9" t="str">
-        <x:v>Tail Light Electrical Connector Corrosion (Mk2)</x:v>
-      </x:c>
-      <x:c r="E32" s="9" t="str">
-        <x:v>Remove tail light assembly, inspect electrical connector for green corrosion. CLEAN connector with electrical contact cleaner and wire brush ($20 DIY). Apply dielectric grease to prevent future corrosion ($10). If connector is severely corroded: Replace pigtail connector ($50-$100 parts). Improve tail light seal with silicone sealant around housing ($15). This is a DIY-friendly repair taking 1-2 hours. If paying shop, costs $150-$300. Address early before corrosion causes shorts.</x:v>
-      </x:c>
-      <x:c r="F32" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G32" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="171.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A33" s="40" t="n">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B33" s="9" t="str">
-        <x:v>audi-tt-water-pump-2008</x:v>
-      </x:c>
-      <x:c r="C33" s="9" t="str">
-        <x:v>2008-2008 | Audi | TT</x:v>
-      </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>C-Pillar Trim Cover Can Detach During Belt-Tensioner Deployment (Recall 08V064)</x:v>
-      </x:c>
-      <x:c r="E33" s="9" t="str">
-        <x:v>Check VIN eligibility. Audi dealers install improved C-pillar trim clips free of charge under recall 08V064.</x:v>
-      </x:c>
-      <x:c r="F33" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G33" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="1161.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A34" s="40" t="n">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="B34" s="9" t="str">
-        <x:v>audi-tts-cam-follower-hpfp-2009</x:v>
-      </x:c>
-      <x:c r="C34" s="9" t="str">
-        <x:v>2009-2015 | Audi | TTS | TTS | EA888</x:v>
-      </x:c>
-      <x:c r="D34" s="9" t="str">
-        <x:v>HPFP Cam Follower Wear and High-Pressure Fuel Pump Failure (Mk2)</x:v>
-      </x:c>
-      <x:c r="E34" s="9" t="str">
-        <x:v>INSPECTION (every 20,000 miles): Remove HPFP (3 bolts) and inspect cam follower surface. If the hardened coating is wearing through (visible copper/brass color), replace follower immediately ($30-$50 part, 30-60 minutes labor). CRITICAL: Ensure cam lobe is at LOW point before reinstalling—if at peak, you'll compress the spring and can break the mounting bolts. If CAMSHAFT WORN (deep groove in lobe): Replace camshaft ($2,000-$4,000). If FUEL PUMP FAILED: Replace HPFP ($400-$800). PREVENTION: Inspect cam follower every 20,000 miles as routine maintenance. Add to every oil change checklist. Consider IE (Integrated Engineering) upgraded HPFP with roller follower to eliminate wear entirely.</x:v>
-      </x:c>
-      <x:c r="F34" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G34" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="884.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A35" s="40" t="n">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B35" s="9" t="str">
-        <x:v>audi-tts-carbon-buildup-2009</x:v>
-      </x:c>
-      <x:c r="C35" s="9" t="str">
-        <x:v>2016-2017 | Audi | TTS</x:v>
-      </x:c>
-      <x:c r="D35" s="9" t="str">
-        <x:v>2016-2017 TTS Cold-Start Misfire DTCs Without Felt Misfire - TSB 2051384/1</x:v>
-      </x:c>
-      <x:c r="E35" s="9" t="str">
-        <x:v>Confirm the exact cold-start timing, simultaneous-cylinder DTC pattern, absence of a felt misfire, CYFB engine and installed ECM software before using this bulletin. When applicable, an Audi-capable workshop updates ECM J623 from software part number 8S0906259C version 0001 to version 0004 or higher using SVM action 01A190, then clears the DTCs. A felt misfire, a different timing or RPM pattern, a different engine/software combination or a returning concern requires normal diagnosis rather than carbon cleaning by assumption.</x:v>
-      </x:c>
-      <x:c r="F35" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G35" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="910.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A36" s="40" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B36" s="9" t="str">
-        <x:v>audi-tts-dsg-mechatronic-2009</x:v>
-      </x:c>
-      <x:c r="C36" s="9" t="str">
-        <x:v>2019-2023 | Audi | TTS</x:v>
-      </x:c>
-      <x:c r="D36" s="9" t="str">
-        <x:v>2019-2023 TTS Clutch K1 Overheat and Transmission DTC Diagnosis - TSB 2060560/3</x:v>
-      </x:c>
-      <x:c r="E36" s="9" t="str">
-        <x:v>Have an Audi-capable workshop check whether TSB 2050723 applies first. If it does not resolve or control the concern, inspect the clutch-K1 maximum-temperature value and document a transmission-fluid sample. Replace the dual clutch, transmission fluid and filter only when the approximately 400 °C K1 value and burnt black or very dark fluid are both present. If those findings are absent, this bulletin does not apply and Audi directs the workshop to continue diagnosis through TAC. Any clutch repair kit must be selected by VIN and production date.</x:v>
-      </x:c>
-      <x:c r="F36" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G36" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="858" hidden="0" customHeight="1">
-      <x:c r="A37" s="40" t="n">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B37" s="9" t="str">
-        <x:v>audi-tts-magnetic-ride-2009</x:v>
-      </x:c>
-      <x:c r="C37" s="9" t="str">
-        <x:v>2016-2016 | Audi | TTS</x:v>
-      </x:c>
-      <x:c r="D37" s="9" t="str">
-        <x:v>2016 TTS Magnetic-Ride Rear Shock-Mount Rumble - TSB 2042539/4</x:v>
-      </x:c>
-      <x:c r="E37" s="9" t="str">
-        <x:v>First reproduce the noise, verify that it comes from the rear shock mounts and confirm that the vehicle was originally equipped with mount 8S0 513 353. Only when those gates are satisfied, remove both rear shock assemblies and replace both mounts with 8V0 513 353 according to Audi workshop instructions, adapt the suspension control position and test drive to confirm the repair. If the installed mount does not match, continue Audi diagnosis. Do not replace magnetic dampers or convert the vehicle to coilovers from this noise alone.</x:v>
-      </x:c>
-      <x:c r="F37" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G37" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="1016.4000244140625" hidden="0" customHeight="1">
-      <x:c r="A38" s="40" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B38" s="9" t="str">
-        <x:v>audi-tts-timing-chain-tensioner-2009</x:v>
-      </x:c>
-      <x:c r="C38" s="9" t="str">
-        <x:v>2009-2015 | Audi | TTS | TTS | EA888 Gen 1, EA888 Gen 2</x:v>
-      </x:c>
-      <x:c r="D38" s="9" t="str">
-        <x:v>Timing Chain Tensioner Failure (EA888 Gen 1/2 - Mk2 TTS)</x:v>
-      </x:c>
-      <x:c r="E38" s="9" t="str">
-        <x:v>PREVENTIVE REPLACEMENT: Replace timing chain, tensioner, guides, and sprockets at 80,000-100,000 miles BEFORE symptoms appear ($2,000-$4,000). This is the MOST important preventive maintenance on the Mk2 TTS. IF RATTLING: Do NOT delay—the chain can jump at any startup. Schedule repair immediately. Use ONLY the latest OEM revised tensioner (06K109467K). IF CHAIN JUMPED: Engine likely destroyed—compression test all cylinders. Rebuild ($5,000-$8,000) or replacement engine ($6,000-$12,000). PREVENTION: Change oil every 5,000 miles with high-quality synthetic. Low oil level accelerates tensioner wear.</x:v>
-      </x:c>
-      <x:c r="F38" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G38" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="976.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A39" s="40" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B39" s="9" t="str">
-        <x:v>audi-tts-water-pump-2009</x:v>
-      </x:c>
-      <x:c r="C39" s="9" t="str">
-        <x:v>2012-2023 | Audi | TTS</x:v>
-      </x:c>
-      <x:c r="D39" s="9" t="str">
-        <x:v>2012 / 2020-2023 TTS Coolant-Pump Update and Leak Diagnosis</x:v>
-      </x:c>
-      <x:c r="E39" s="9" t="str">
-        <x:v>For a 2012 TTS, ask an Audi dealer to check the VIN and current campaign/action history for Update 19J2; the published update replaced the pump only when its exact criteria were met and does not promise current warranty coverage. For a 2020-2023 2.0L TTS, first exclude a low level caused by incomplete bleeding or an earlier repair, document and clean the suspected leak, refill to maximum and recheck after driving. Continue observation when no leak returns; replace only the component proven to leak when coolant reappears. Do not select a pump or thermostat assembly before VIN-, engine- and leak-specific diagnosis.</x:v>
-      </x:c>
-      <x:c r="F39" s="9" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G39" s="41" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="198" hidden="0" customHeight="1">
-      <x:c r="A40" s="42" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B40" s="43" t="str">
-        <x:v>audi-tts-waterpump-housing-2009</x:v>
-      </x:c>
-      <x:c r="C40" s="43" t="str">
-        <x:v>2009-2024 | Audi | TTS | EA888</x:v>
-      </x:c>
-      <x:c r="D40" s="43" t="str">
-        <x:v>Water Pump and Thermostat Housing Failure</x:v>
-      </x:c>
-      <x:c r="E40" s="43" t="str">
-        <x:v>Replace water pump, thermostat, and housing as a complete assembly. Use metal-impeller aftermarket pump if available.</x:v>
-      </x:c>
-      <x:c r="F40" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G40" s="44" t="str">
-        <x:v>PENDING REPAIR-FIRST REVIEW</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -22574,7 +24034,7 @@
       <x:c r="F2" s="28"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="45" t="str">
+      <x:c r="A3" s="48" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
@@ -22586,7 +24046,7 @@
       <x:c r="F3" s="28"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="45" t="str">
+      <x:c r="A4" s="48" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="15" t="str">
@@ -22598,7 +24058,7 @@
       <x:c r="F4" s="28"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="45" t="str">
+      <x:c r="A5" s="48" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
@@ -22610,7 +24070,7 @@
       <x:c r="F5" s="28"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="45" t="str">
+      <x:c r="A6" s="48" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
@@ -22622,7 +24082,7 @@
       <x:c r="F6" s="28"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="45" t="str">
+      <x:c r="A7" s="48" t="str">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
@@ -22634,7 +24094,7 @@
       <x:c r="F7" s="28"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="45" t="str">
+      <x:c r="A8" s="48" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
@@ -22646,7 +24106,7 @@
       <x:c r="F8" s="28"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="45" t="str">
+      <x:c r="A9" s="48" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
@@ -22658,7 +24118,7 @@
       <x:c r="F9" s="28"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="45" t="str">
+      <x:c r="A10" s="48" t="str">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
@@ -22678,7 +24138,7 @@
       <x:c r="F11" s="28"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="46" t="str">
+      <x:c r="A12" s="49" t="str">
         <x:v>Artifact state</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
@@ -22690,7 +24150,7 @@
       <x:c r="F12" s="28"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="46" t="str">
+      <x:c r="A13" s="49" t="str">
         <x:v>Source</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
@@ -22702,7 +24162,7 @@
       <x:c r="F13" s="28"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="46" t="str">
+      <x:c r="A14" s="49" t="str">
         <x:v>Review input</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
@@ -22714,16 +24174,16 @@
       <x:c r="F14" s="28"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="47" t="str">
+      <x:c r="A15" s="50" t="str">
         <x:v>Generated ledger</x:v>
       </x:c>
-      <x:c r="B15" s="48" t="str">
+      <x:c r="B15" s="51" t="str">
         <x:v>data\audi-repair-first-review\review-ledger.json</x:v>
       </x:c>
-      <x:c r="C15" s="48"/>
-      <x:c r="D15" s="48"/>
-      <x:c r="E15" s="48"/>
-      <x:c r="F15" s="49"/>
+      <x:c r="C15" s="51"/>
+      <x:c r="D15" s="51"/>
+      <x:c r="E15" s="51"/>
+      <x:c r="F15" s="52"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>